<commit_message>
Katalog guncellendi - 19.01.2026 10:24:57,70
</commit_message>
<xml_diff>
--- a/urunler.xlsx
+++ b/urunler.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/49dd5535ee0ab452/Desktop/CEREN-PC/SIVAL_GIYIM_KATALOG/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="194" documentId="13_ncr:1_{CCE8B614-DB69-4334-AC06-D714AC841E42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2B541A64-EA0F-4DCC-A056-87AD91AE2D16}"/>
+  <xr:revisionPtr revIDLastSave="200" documentId="13_ncr:1_{CCE8B614-DB69-4334-AC06-D714AC841E42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6CCB6A72-3E60-4DF3-AF20-E3F47A40E665}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -64,9 +64,6 @@
     <t>300 TL</t>
   </si>
   <si>
-    <t xml:space="preserve">300 TL </t>
-  </si>
-  <si>
     <t>BAG6.jpg</t>
   </si>
   <si>
@@ -983,6 +980,9 @@
   </si>
   <si>
     <t>243-2.jpg</t>
+  </si>
+  <si>
+    <t>350TL</t>
   </si>
 </sst>
 </file>
@@ -1412,7 +1412,7 @@
         <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>320</v>
       </c>
       <c r="C2" t="s">
         <v>7</v>
@@ -1421,7 +1421,7 @@
         <v>8</v>
       </c>
       <c r="E2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F2" t="s">
         <v>6</v>
@@ -1432,7 +1432,7 @@
         <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>320</v>
       </c>
       <c r="C3" t="s">
         <v>7</v>
@@ -1441,7 +1441,7 @@
         <v>9</v>
       </c>
       <c r="E3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F3" t="s">
         <v>6</v>
@@ -1452,36 +1452,36 @@
         <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>320</v>
       </c>
       <c r="C4" t="s">
         <v>7</v>
       </c>
       <c r="D4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E4" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F4" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>320</v>
       </c>
       <c r="C5" t="s">
         <v>7</v>
       </c>
       <c r="D5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F5" t="s">
         <v>6</v>
@@ -1489,19 +1489,19 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B6" t="s">
-        <v>13</v>
+        <v>320</v>
       </c>
       <c r="C6" t="s">
         <v>7</v>
       </c>
       <c r="D6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E6" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F6" t="s">
         <v>6</v>
@@ -1509,19 +1509,19 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B7" t="s">
-        <v>13</v>
+        <v>320</v>
       </c>
       <c r="C7" t="s">
         <v>7</v>
       </c>
       <c r="D7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E7" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F7" t="s">
         <v>6</v>
@@ -1529,39 +1529,39 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B8" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C8" t="s">
         <v>7</v>
       </c>
       <c r="D8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B9" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C9" t="s">
         <v>7</v>
       </c>
       <c r="D9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F9" t="s">
         <v>6</v>
@@ -1569,19 +1569,19 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B10" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C10" t="s">
         <v>7</v>
       </c>
       <c r="D10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F10" t="s">
         <v>6</v>
@@ -1589,19 +1589,19 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B11" t="s">
         <v>13</v>
       </c>
       <c r="C11" t="s">
+        <v>27</v>
+      </c>
+      <c r="D11" t="s">
         <v>28</v>
       </c>
-      <c r="D11" t="s">
-        <v>29</v>
-      </c>
       <c r="E11" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F11" t="s">
         <v>6</v>
@@ -1609,39 +1609,39 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B12" t="s">
         <v>13</v>
       </c>
       <c r="C12" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D12" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E12" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F12" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B13" t="s">
         <v>13</v>
       </c>
       <c r="C13" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E13" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F13" t="s">
         <v>6</v>
@@ -1649,19 +1649,19 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B14" t="s">
         <v>13</v>
       </c>
       <c r="C14" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D14" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E14" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F14" t="s">
         <v>6</v>
@@ -1669,19 +1669,19 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B15" t="s">
         <v>13</v>
       </c>
       <c r="C15" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D15" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E15" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F15" t="s">
         <v>6</v>
@@ -1689,19 +1689,19 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B16" t="s">
         <v>13</v>
       </c>
       <c r="C16" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D16" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E16" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F16" t="s">
         <v>6</v>
@@ -1709,19 +1709,19 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B17" t="s">
         <v>13</v>
       </c>
       <c r="C17" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D17" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E17" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F17" t="s">
         <v>6</v>
@@ -1729,19 +1729,19 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B18" t="s">
         <v>13</v>
       </c>
       <c r="C18" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D18" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E18" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F18" t="s">
         <v>6</v>
@@ -1749,19 +1749,19 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B19" t="s">
         <v>13</v>
       </c>
       <c r="C19" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D19" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E19" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F19" t="s">
         <v>6</v>
@@ -1769,19 +1769,19 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B20" t="s">
         <v>13</v>
       </c>
       <c r="C20" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D20" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E20" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F20" t="s">
         <v>6</v>
@@ -1789,19 +1789,19 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B21" t="s">
         <v>13</v>
       </c>
       <c r="C21" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D21" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E21" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F21" t="s">
         <v>6</v>
@@ -1809,19 +1809,19 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B22" t="s">
         <v>13</v>
       </c>
       <c r="C22" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D22" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E22" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F22" t="s">
         <v>6</v>
@@ -1829,19 +1829,19 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B23" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C23" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D23" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E23" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F23" t="s">
         <v>6</v>
@@ -1849,19 +1849,19 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>55</v>
+      </c>
+      <c r="B24" t="s">
+        <v>126</v>
+      </c>
+      <c r="C24" t="s">
+        <v>27</v>
+      </c>
+      <c r="D24" t="s">
         <v>56</v>
       </c>
-      <c r="B24" t="s">
-        <v>127</v>
-      </c>
-      <c r="C24" t="s">
-        <v>28</v>
-      </c>
-      <c r="D24" t="s">
-        <v>57</v>
-      </c>
       <c r="E24" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F24" t="s">
         <v>6</v>
@@ -1869,19 +1869,19 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>57</v>
+      </c>
+      <c r="B25" t="s">
+        <v>126</v>
+      </c>
+      <c r="C25" t="s">
+        <v>27</v>
+      </c>
+      <c r="D25" t="s">
         <v>58</v>
       </c>
-      <c r="B25" t="s">
-        <v>127</v>
-      </c>
-      <c r="C25" t="s">
-        <v>28</v>
-      </c>
-      <c r="D25" t="s">
-        <v>59</v>
-      </c>
       <c r="E25" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F25" t="s">
         <v>6</v>
@@ -1889,19 +1889,19 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B26" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C26" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D26" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F26" t="s">
         <v>6</v>
@@ -1909,19 +1909,19 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>61</v>
+      </c>
+      <c r="B27" t="s">
+        <v>127</v>
+      </c>
+      <c r="C27" t="s">
+        <v>27</v>
+      </c>
+      <c r="D27" t="s">
         <v>62</v>
       </c>
-      <c r="B27" t="s">
-        <v>128</v>
-      </c>
-      <c r="C27" t="s">
-        <v>28</v>
-      </c>
-      <c r="D27" t="s">
-        <v>63</v>
-      </c>
       <c r="E27" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F27" t="s">
         <v>6</v>
@@ -1929,19 +1929,19 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
+        <v>63</v>
+      </c>
+      <c r="B28" t="s">
+        <v>127</v>
+      </c>
+      <c r="C28" t="s">
+        <v>27</v>
+      </c>
+      <c r="D28" t="s">
         <v>64</v>
       </c>
-      <c r="B28" t="s">
-        <v>128</v>
-      </c>
-      <c r="C28" t="s">
-        <v>28</v>
-      </c>
-      <c r="D28" t="s">
-        <v>65</v>
-      </c>
       <c r="E28" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F28" t="s">
         <v>6</v>
@@ -1949,19 +1949,19 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>65</v>
+      </c>
+      <c r="B29" t="s">
+        <v>127</v>
+      </c>
+      <c r="C29" t="s">
+        <v>27</v>
+      </c>
+      <c r="D29" t="s">
         <v>66</v>
       </c>
-      <c r="B29" t="s">
-        <v>128</v>
-      </c>
-      <c r="C29" t="s">
-        <v>28</v>
-      </c>
-      <c r="D29" t="s">
-        <v>67</v>
-      </c>
       <c r="E29" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F29" t="s">
         <v>6</v>
@@ -1969,19 +1969,19 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B30" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C30" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D30" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F30" t="s">
         <v>6</v>
@@ -1989,19 +1989,19 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B31" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C31" t="s">
         <v>7</v>
       </c>
       <c r="D31" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F31" t="s">
         <v>6</v>
@@ -2009,19 +2009,19 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B32" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C32" t="s">
         <v>7</v>
       </c>
       <c r="D32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F32" t="s">
         <v>6</v>
@@ -2029,19 +2029,19 @@
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B33" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C33" t="s">
         <v>7</v>
       </c>
       <c r="D33" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F33" t="s">
         <v>6</v>
@@ -2049,19 +2049,19 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B34" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C34" t="s">
         <v>7</v>
       </c>
       <c r="D34" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F34" t="s">
         <v>6</v>
@@ -2069,19 +2069,19 @@
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B35" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C35" t="s">
         <v>7</v>
       </c>
       <c r="D35" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F35" t="s">
         <v>6</v>
@@ -2089,19 +2089,19 @@
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B36" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C36" t="s">
         <v>7</v>
       </c>
       <c r="D36" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F36" t="s">
         <v>6</v>
@@ -2109,19 +2109,19 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B37" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C37" t="s">
         <v>7</v>
       </c>
       <c r="D37" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F37" t="s">
         <v>6</v>
@@ -2129,19 +2129,19 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B38" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C38" t="s">
         <v>7</v>
       </c>
       <c r="D38" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="F38" t="s">
         <v>6</v>
@@ -2149,19 +2149,19 @@
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B39" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C39" t="s">
         <v>7</v>
       </c>
       <c r="D39" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="F39" t="s">
         <v>6</v>
@@ -2169,19 +2169,19 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B40" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C40" t="s">
         <v>7</v>
       </c>
       <c r="D40" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="F40" t="s">
         <v>6</v>
@@ -2189,19 +2189,19 @@
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B41" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C41" t="s">
         <v>7</v>
       </c>
       <c r="D41" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="F41" t="s">
         <v>6</v>
@@ -2209,19 +2209,19 @@
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B42" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C42" t="s">
         <v>7</v>
       </c>
       <c r="D42" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="F42" t="s">
         <v>6</v>
@@ -2229,19 +2229,19 @@
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B43" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C43" t="s">
         <v>7</v>
       </c>
       <c r="D43" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="F43" t="s">
         <v>6</v>
@@ -2249,19 +2249,19 @@
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B44" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C44" t="s">
         <v>7</v>
       </c>
       <c r="D44" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="F44" t="s">
         <v>6</v>
@@ -2269,19 +2269,19 @@
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B45" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C45" t="s">
         <v>7</v>
       </c>
       <c r="D45" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="F45" t="s">
         <v>6</v>
@@ -2289,19 +2289,19 @@
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B46" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C46" t="s">
         <v>7</v>
       </c>
       <c r="D46" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="F46" t="s">
         <v>6</v>
@@ -2309,19 +2309,19 @@
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B47" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C47" t="s">
         <v>7</v>
       </c>
       <c r="D47" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="F47" t="s">
         <v>6</v>
@@ -2329,19 +2329,19 @@
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B48" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C48" t="s">
         <v>7</v>
       </c>
       <c r="D48" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="F48" t="s">
         <v>6</v>
@@ -2349,19 +2349,19 @@
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B49" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C49" t="s">
         <v>7</v>
       </c>
       <c r="D49" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F49" t="s">
         <v>6</v>
@@ -2369,19 +2369,19 @@
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B50" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C50" t="s">
         <v>7</v>
       </c>
       <c r="D50" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F50" t="s">
         <v>6</v>
@@ -2389,19 +2389,19 @@
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B51" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C51" t="s">
         <v>7</v>
       </c>
       <c r="D51" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F51" t="s">
         <v>6</v>
@@ -2409,19 +2409,19 @@
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B52" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C52" t="s">
         <v>7</v>
       </c>
       <c r="D52" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F52" t="s">
         <v>6</v>
@@ -2429,19 +2429,19 @@
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
+        <v>112</v>
+      </c>
+      <c r="B53" t="s">
+        <v>129</v>
+      </c>
+      <c r="C53" t="s">
         <v>113</v>
       </c>
-      <c r="B53" t="s">
-        <v>130</v>
-      </c>
-      <c r="C53" t="s">
+      <c r="D53" t="s">
+        <v>137</v>
+      </c>
+      <c r="E53" t="s">
         <v>114</v>
-      </c>
-      <c r="D53" t="s">
-        <v>138</v>
-      </c>
-      <c r="E53" t="s">
-        <v>115</v>
       </c>
       <c r="F53" t="s">
         <v>6</v>
@@ -2449,19 +2449,19 @@
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
+        <v>115</v>
+      </c>
+      <c r="B54" t="s">
+        <v>129</v>
+      </c>
+      <c r="C54" t="s">
+        <v>113</v>
+      </c>
+      <c r="D54" t="s">
         <v>116</v>
       </c>
-      <c r="B54" t="s">
-        <v>130</v>
-      </c>
-      <c r="C54" t="s">
+      <c r="E54" t="s">
         <v>114</v>
-      </c>
-      <c r="D54" t="s">
-        <v>117</v>
-      </c>
-      <c r="E54" t="s">
-        <v>115</v>
       </c>
       <c r="F54" t="s">
         <v>6</v>
@@ -2469,19 +2469,19 @@
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
+        <v>117</v>
+      </c>
+      <c r="B55" t="s">
+        <v>129</v>
+      </c>
+      <c r="C55" t="s">
+        <v>113</v>
+      </c>
+      <c r="D55" t="s">
         <v>118</v>
       </c>
-      <c r="B55" t="s">
-        <v>130</v>
-      </c>
-      <c r="C55" t="s">
+      <c r="E55" t="s">
         <v>114</v>
-      </c>
-      <c r="D55" t="s">
-        <v>119</v>
-      </c>
-      <c r="E55" t="s">
-        <v>115</v>
       </c>
       <c r="F55" t="s">
         <v>6</v>
@@ -2489,19 +2489,19 @@
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B56" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C56" t="s">
         <v>7</v>
       </c>
       <c r="D56" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E56" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F56" t="s">
         <v>6</v>
@@ -2509,19 +2509,19 @@
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B57" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C57" t="s">
         <v>7</v>
       </c>
       <c r="D57" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E57" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F57" t="s">
         <v>6</v>
@@ -2529,219 +2529,219 @@
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
+        <v>138</v>
+      </c>
+      <c r="B58" t="s">
         <v>139</v>
       </c>
-      <c r="B58" t="s">
+      <c r="C58" t="s">
+        <v>113</v>
+      </c>
+      <c r="D58" t="s">
+        <v>141</v>
+      </c>
+      <c r="E58" t="s">
         <v>140</v>
       </c>
-      <c r="C58" t="s">
-        <v>114</v>
-      </c>
-      <c r="D58" t="s">
-        <v>142</v>
-      </c>
-      <c r="E58" t="s">
-        <v>141</v>
-      </c>
       <c r="F58" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B59" t="s">
+        <v>139</v>
+      </c>
+      <c r="C59" t="s">
+        <v>113</v>
+      </c>
+      <c r="D59" t="s">
+        <v>142</v>
+      </c>
+      <c r="E59" t="s">
         <v>140</v>
       </c>
-      <c r="C59" t="s">
-        <v>114</v>
-      </c>
-      <c r="D59" t="s">
-        <v>143</v>
-      </c>
-      <c r="E59" t="s">
-        <v>141</v>
-      </c>
       <c r="F59" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B60" t="s">
+        <v>139</v>
+      </c>
+      <c r="C60" t="s">
+        <v>113</v>
+      </c>
+      <c r="D60" t="s">
+        <v>144</v>
+      </c>
+      <c r="E60" t="s">
         <v>140</v>
       </c>
-      <c r="C60" t="s">
-        <v>114</v>
-      </c>
-      <c r="D60" t="s">
-        <v>145</v>
-      </c>
-      <c r="E60" t="s">
-        <v>141</v>
-      </c>
       <c r="F60" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B61" t="s">
+        <v>139</v>
+      </c>
+      <c r="C61" t="s">
+        <v>113</v>
+      </c>
+      <c r="D61" t="s">
+        <v>146</v>
+      </c>
+      <c r="E61" t="s">
         <v>140</v>
       </c>
-      <c r="C61" t="s">
-        <v>114</v>
-      </c>
-      <c r="D61" t="s">
-        <v>147</v>
-      </c>
-      <c r="E61" t="s">
-        <v>141</v>
-      </c>
       <c r="F61" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B62" t="s">
+        <v>139</v>
+      </c>
+      <c r="C62" t="s">
+        <v>113</v>
+      </c>
+      <c r="D62" t="s">
+        <v>148</v>
+      </c>
+      <c r="E62" t="s">
         <v>140</v>
       </c>
-      <c r="C62" t="s">
-        <v>114</v>
-      </c>
-      <c r="D62" t="s">
-        <v>149</v>
-      </c>
-      <c r="E62" t="s">
-        <v>141</v>
-      </c>
       <c r="F62" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B63" t="s">
+        <v>139</v>
+      </c>
+      <c r="C63" t="s">
+        <v>113</v>
+      </c>
+      <c r="D63" t="s">
+        <v>150</v>
+      </c>
+      <c r="E63" t="s">
         <v>140</v>
       </c>
-      <c r="C63" t="s">
-        <v>114</v>
-      </c>
-      <c r="D63" t="s">
-        <v>151</v>
-      </c>
-      <c r="E63" t="s">
-        <v>141</v>
-      </c>
       <c r="F63" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
+        <v>152</v>
+      </c>
+      <c r="B64" t="s">
+        <v>154</v>
+      </c>
+      <c r="C64" t="s">
+        <v>113</v>
+      </c>
+      <c r="D64" t="s">
         <v>153</v>
       </c>
-      <c r="B64" t="s">
-        <v>155</v>
-      </c>
-      <c r="C64" t="s">
-        <v>114</v>
-      </c>
-      <c r="D64" t="s">
-        <v>154</v>
-      </c>
       <c r="E64" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F64" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B65" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C65" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D65" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E65" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F65" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B66" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C66" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D66" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E66" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F66" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B67" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C67" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D67" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="E67" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F67" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
+        <v>160</v>
+      </c>
+      <c r="B68" t="s">
         <v>161</v>
       </c>
-      <c r="B68" t="s">
-        <v>162</v>
-      </c>
       <c r="C68" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D68" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="E68" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F68" t="s">
         <v>6</v>
@@ -2749,119 +2749,119 @@
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B69" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C69" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D69" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E69" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F69" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
+        <v>166</v>
+      </c>
+      <c r="B70" t="s">
         <v>167</v>
       </c>
-      <c r="B70" t="s">
-        <v>168</v>
-      </c>
       <c r="C70" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D70" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E70" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F70" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B71" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C71" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D71" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E71" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F71" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B72" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C72" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D72" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E72" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F72" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
+        <v>173</v>
+      </c>
+      <c r="B73" t="s">
         <v>174</v>
       </c>
-      <c r="B73" t="s">
-        <v>175</v>
-      </c>
       <c r="C73" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D73" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E73" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F73" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B74" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C74" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D74" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E74" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F74" t="s">
         <v>6</v>
@@ -2869,19 +2869,19 @@
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B75" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C75" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D75" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E75" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F75" t="s">
         <v>6</v>
@@ -2889,19 +2889,19 @@
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B76" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C76" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D76" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E76" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F76" t="s">
         <v>6</v>
@@ -2909,19 +2909,19 @@
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B77" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C77" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D77" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E77" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F77" t="s">
         <v>6</v>
@@ -2929,19 +2929,19 @@
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B78" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C78" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D78" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="E78" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F78" t="s">
         <v>6</v>
@@ -2949,19 +2949,19 @@
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
+        <v>190</v>
+      </c>
+      <c r="B79" t="s">
+        <v>126</v>
+      </c>
+      <c r="C79" t="s">
         <v>191</v>
       </c>
-      <c r="B79" t="s">
-        <v>127</v>
-      </c>
-      <c r="C79" t="s">
-        <v>192</v>
-      </c>
       <c r="D79" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="E79" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F79" t="s">
         <v>6</v>
@@ -2969,19 +2969,19 @@
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
+        <v>192</v>
+      </c>
+      <c r="B80" t="s">
         <v>193</v>
       </c>
-      <c r="B80" t="s">
+      <c r="C80" t="s">
+        <v>191</v>
+      </c>
+      <c r="D80" t="s">
         <v>194</v>
       </c>
-      <c r="C80" t="s">
-        <v>192</v>
-      </c>
-      <c r="D80" t="s">
-        <v>195</v>
-      </c>
       <c r="E80" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F80" t="s">
         <v>6</v>
@@ -2989,19 +2989,19 @@
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B81" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C81" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D81" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E81" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F81" t="s">
         <v>6</v>
@@ -3009,19 +3009,19 @@
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
+        <v>197</v>
+      </c>
+      <c r="B82" t="s">
+        <v>193</v>
+      </c>
+      <c r="C82" t="s">
+        <v>191</v>
+      </c>
+      <c r="D82" t="s">
         <v>198</v>
       </c>
-      <c r="B82" t="s">
-        <v>194</v>
-      </c>
-      <c r="C82" t="s">
-        <v>192</v>
-      </c>
-      <c r="D82" t="s">
-        <v>199</v>
-      </c>
       <c r="E82" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F82" t="s">
         <v>6</v>
@@ -3029,19 +3029,19 @@
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
+        <v>199</v>
+      </c>
+      <c r="B83" t="s">
+        <v>193</v>
+      </c>
+      <c r="C83" t="s">
+        <v>191</v>
+      </c>
+      <c r="D83" t="s">
         <v>200</v>
       </c>
-      <c r="B83" t="s">
-        <v>194</v>
-      </c>
-      <c r="C83" t="s">
-        <v>192</v>
-      </c>
-      <c r="D83" t="s">
-        <v>201</v>
-      </c>
       <c r="E83" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F83" t="s">
         <v>6</v>
@@ -3049,19 +3049,19 @@
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B84" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C84" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D84" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="E84" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F84" t="s">
         <v>6</v>
@@ -3069,19 +3069,19 @@
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B85" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C85" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D85" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="E85" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F85" t="s">
         <v>6</v>
@@ -3089,19 +3089,19 @@
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B86" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C86" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D86" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E86" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F86" t="s">
         <v>6</v>
@@ -3109,19 +3109,19 @@
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
+        <v>209</v>
+      </c>
+      <c r="B87" t="s">
+        <v>193</v>
+      </c>
+      <c r="C87" t="s">
+        <v>191</v>
+      </c>
+      <c r="D87" t="s">
+        <v>205</v>
+      </c>
+      <c r="E87" t="s">
         <v>210</v>
-      </c>
-      <c r="B87" t="s">
-        <v>194</v>
-      </c>
-      <c r="C87" t="s">
-        <v>192</v>
-      </c>
-      <c r="D87" t="s">
-        <v>206</v>
-      </c>
-      <c r="E87" t="s">
-        <v>211</v>
       </c>
       <c r="F87" t="s">
         <v>6</v>
@@ -3129,19 +3129,19 @@
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B88" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C88" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D88" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E88" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F88" t="s">
         <v>6</v>
@@ -3149,19 +3149,19 @@
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
+        <v>211</v>
+      </c>
+      <c r="B89" t="s">
         <v>212</v>
       </c>
-      <c r="B89" t="s">
+      <c r="C89" t="s">
         <v>213</v>
       </c>
-      <c r="C89" t="s">
+      <c r="D89" t="s">
         <v>214</v>
       </c>
-      <c r="D89" t="s">
+      <c r="E89" t="s">
         <v>215</v>
-      </c>
-      <c r="E89" t="s">
-        <v>216</v>
       </c>
       <c r="F89" t="s">
         <v>6</v>
@@ -3169,19 +3169,19 @@
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B90" t="s">
+        <v>212</v>
+      </c>
+      <c r="C90" t="s">
         <v>213</v>
       </c>
-      <c r="C90" t="s">
-        <v>214</v>
-      </c>
       <c r="D90" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="E90" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F90" t="s">
         <v>6</v>
@@ -3189,19 +3189,19 @@
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B91" t="s">
+        <v>212</v>
+      </c>
+      <c r="C91" t="s">
         <v>213</v>
       </c>
-      <c r="C91" t="s">
-        <v>214</v>
-      </c>
       <c r="D91" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="E91" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F91" t="s">
         <v>6</v>
@@ -3209,19 +3209,19 @@
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B92" t="s">
+        <v>212</v>
+      </c>
+      <c r="C92" t="s">
         <v>213</v>
       </c>
-      <c r="C92" t="s">
-        <v>214</v>
-      </c>
       <c r="D92" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="E92" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F92" t="s">
         <v>6</v>
@@ -3229,19 +3229,19 @@
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B93" t="s">
+        <v>212</v>
+      </c>
+      <c r="C93" t="s">
         <v>213</v>
       </c>
-      <c r="C93" t="s">
-        <v>214</v>
-      </c>
       <c r="D93" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="E93" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F93" t="s">
         <v>6</v>
@@ -3249,19 +3249,19 @@
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B94" t="s">
+        <v>212</v>
+      </c>
+      <c r="C94" t="s">
         <v>213</v>
       </c>
-      <c r="C94" t="s">
-        <v>214</v>
-      </c>
       <c r="D94" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E94" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F94" t="s">
         <v>6</v>
@@ -3269,19 +3269,19 @@
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B95" t="s">
+        <v>212</v>
+      </c>
+      <c r="C95" t="s">
         <v>213</v>
       </c>
-      <c r="C95" t="s">
-        <v>214</v>
-      </c>
       <c r="D95" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="E95" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F95" t="s">
         <v>6</v>
@@ -3289,19 +3289,19 @@
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B96" t="s">
+        <v>212</v>
+      </c>
+      <c r="C96" t="s">
         <v>213</v>
       </c>
-      <c r="C96" t="s">
-        <v>214</v>
-      </c>
       <c r="D96" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E96" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F96" t="s">
         <v>6</v>
@@ -3309,19 +3309,19 @@
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B97" t="s">
+        <v>212</v>
+      </c>
+      <c r="C97" t="s">
         <v>213</v>
       </c>
-      <c r="C97" t="s">
-        <v>214</v>
-      </c>
       <c r="D97" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E97" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F97" t="s">
         <v>6</v>
@@ -3329,19 +3329,19 @@
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
+        <v>232</v>
+      </c>
+      <c r="B98" t="s">
+        <v>126</v>
+      </c>
+      <c r="C98" t="s">
+        <v>213</v>
+      </c>
+      <c r="D98" t="s">
         <v>233</v>
       </c>
-      <c r="B98" t="s">
-        <v>127</v>
-      </c>
-      <c r="C98" t="s">
-        <v>214</v>
-      </c>
-      <c r="D98" t="s">
-        <v>234</v>
-      </c>
       <c r="E98" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F98" t="s">
         <v>6</v>
@@ -3349,19 +3349,19 @@
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B99" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C99" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D99" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E99" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F99" t="s">
         <v>6</v>
@@ -3369,19 +3369,19 @@
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B100" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C100" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D100" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E100" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F100" t="s">
         <v>6</v>
@@ -3389,19 +3389,19 @@
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
+        <v>236</v>
+      </c>
+      <c r="B101" t="s">
         <v>237</v>
       </c>
-      <c r="B101" t="s">
+      <c r="C101" t="s">
+        <v>191</v>
+      </c>
+      <c r="D101" t="s">
         <v>238</v>
       </c>
-      <c r="C101" t="s">
-        <v>192</v>
-      </c>
-      <c r="D101" t="s">
-        <v>239</v>
-      </c>
       <c r="E101" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F101" t="s">
         <v>6</v>
@@ -3409,19 +3409,19 @@
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B102" t="s">
+        <v>239</v>
+      </c>
+      <c r="C102" t="s">
+        <v>191</v>
+      </c>
+      <c r="D102" t="s">
         <v>240</v>
       </c>
-      <c r="C102" t="s">
-        <v>192</v>
-      </c>
-      <c r="D102" t="s">
-        <v>241</v>
-      </c>
       <c r="E102" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F102" t="s">
         <v>6</v>
@@ -3429,19 +3429,19 @@
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B103" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C103" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D103" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="E103" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F103" t="s">
         <v>6</v>
@@ -3449,19 +3449,19 @@
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B104" t="s">
+        <v>247</v>
+      </c>
+      <c r="C104" t="s">
+        <v>191</v>
+      </c>
+      <c r="D104" t="s">
         <v>248</v>
       </c>
-      <c r="C104" t="s">
-        <v>192</v>
-      </c>
-      <c r="D104" t="s">
-        <v>249</v>
-      </c>
       <c r="E104" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F104" t="s">
         <v>6</v>
@@ -3469,19 +3469,19 @@
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
+        <v>246</v>
+      </c>
+      <c r="B105" t="s">
         <v>247</v>
       </c>
-      <c r="B105" t="s">
-        <v>248</v>
-      </c>
       <c r="C105" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D105" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="E105" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F105" t="s">
         <v>6</v>
@@ -3489,19 +3489,19 @@
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B106" t="s">
+        <v>250</v>
+      </c>
+      <c r="C106" t="s">
         <v>251</v>
       </c>
-      <c r="C106" t="s">
+      <c r="D106" t="s">
         <v>252</v>
       </c>
-      <c r="D106" t="s">
-        <v>253</v>
-      </c>
       <c r="E106" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="F106" t="s">
         <v>6</v>
@@ -3509,19 +3509,19 @@
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B107" t="s">
+        <v>250</v>
+      </c>
+      <c r="C107" t="s">
         <v>251</v>
       </c>
-      <c r="C107" t="s">
-        <v>252</v>
-      </c>
       <c r="D107" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="E107" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="F107" t="s">
         <v>6</v>
@@ -3529,19 +3529,19 @@
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B108" t="s">
+        <v>250</v>
+      </c>
+      <c r="C108" t="s">
         <v>251</v>
       </c>
-      <c r="C108" t="s">
-        <v>252</v>
-      </c>
       <c r="D108" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E108" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="F108" t="s">
         <v>6</v>
@@ -3549,19 +3549,19 @@
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
+        <v>259</v>
+      </c>
+      <c r="B109" t="s">
+        <v>250</v>
+      </c>
+      <c r="C109" t="s">
+        <v>251</v>
+      </c>
+      <c r="D109" t="s">
+        <v>258</v>
+      </c>
+      <c r="E109" t="s">
         <v>260</v>
-      </c>
-      <c r="B109" t="s">
-        <v>251</v>
-      </c>
-      <c r="C109" t="s">
-        <v>252</v>
-      </c>
-      <c r="D109" t="s">
-        <v>259</v>
-      </c>
-      <c r="E109" t="s">
-        <v>261</v>
       </c>
       <c r="F109" t="s">
         <v>6</v>
@@ -3569,19 +3569,19 @@
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
+        <v>261</v>
+      </c>
+      <c r="B110" t="s">
+        <v>126</v>
+      </c>
+      <c r="C110" t="s">
+        <v>251</v>
+      </c>
+      <c r="D110" t="s">
         <v>262</v>
       </c>
-      <c r="B110" t="s">
-        <v>127</v>
-      </c>
-      <c r="C110" t="s">
-        <v>252</v>
-      </c>
-      <c r="D110" t="s">
-        <v>263</v>
-      </c>
       <c r="E110" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="F110" t="s">
         <v>6</v>
@@ -3589,19 +3589,19 @@
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
+        <v>263</v>
+      </c>
+      <c r="B111" t="s">
+        <v>126</v>
+      </c>
+      <c r="C111" t="s">
+        <v>251</v>
+      </c>
+      <c r="D111" t="s">
         <v>264</v>
       </c>
-      <c r="B111" t="s">
-        <v>127</v>
-      </c>
-      <c r="C111" t="s">
-        <v>252</v>
-      </c>
-      <c r="D111" t="s">
-        <v>265</v>
-      </c>
       <c r="E111" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="F111" t="s">
         <v>6</v>
@@ -3609,19 +3609,19 @@
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
+        <v>265</v>
+      </c>
+      <c r="B112" t="s">
+        <v>126</v>
+      </c>
+      <c r="C112" t="s">
+        <v>251</v>
+      </c>
+      <c r="D112" t="s">
         <v>266</v>
       </c>
-      <c r="B112" t="s">
-        <v>127</v>
-      </c>
-      <c r="C112" t="s">
-        <v>252</v>
-      </c>
-      <c r="D112" t="s">
-        <v>267</v>
-      </c>
       <c r="E112" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="F112" t="s">
         <v>6</v>
@@ -3629,19 +3629,19 @@
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B113" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C113" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D113" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="E113" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="F113" t="s">
         <v>6</v>
@@ -3649,19 +3649,19 @@
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
+        <v>268</v>
+      </c>
+      <c r="B114" t="s">
+        <v>126</v>
+      </c>
+      <c r="C114" t="s">
+        <v>251</v>
+      </c>
+      <c r="D114" t="s">
         <v>269</v>
       </c>
-      <c r="B114" t="s">
-        <v>127</v>
-      </c>
-      <c r="C114" t="s">
-        <v>252</v>
-      </c>
-      <c r="D114" t="s">
-        <v>270</v>
-      </c>
       <c r="E114" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="F114" t="s">
         <v>6</v>
@@ -3669,19 +3669,19 @@
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
+        <v>275</v>
+      </c>
+      <c r="B115" t="s">
+        <v>271</v>
+      </c>
+      <c r="C115" t="s">
+        <v>27</v>
+      </c>
+      <c r="D115" t="s">
         <v>276</v>
       </c>
-      <c r="B115" t="s">
+      <c r="E115" t="s">
         <v>272</v>
-      </c>
-      <c r="C115" t="s">
-        <v>28</v>
-      </c>
-      <c r="D115" t="s">
-        <v>277</v>
-      </c>
-      <c r="E115" t="s">
-        <v>273</v>
       </c>
       <c r="F115" t="s">
         <v>6</v>
@@ -3689,19 +3689,19 @@
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B116" t="s">
+        <v>271</v>
+      </c>
+      <c r="C116" t="s">
+        <v>27</v>
+      </c>
+      <c r="D116" t="s">
+        <v>277</v>
+      </c>
+      <c r="E116" t="s">
         <v>272</v>
-      </c>
-      <c r="C116" t="s">
-        <v>28</v>
-      </c>
-      <c r="D116" t="s">
-        <v>278</v>
-      </c>
-      <c r="E116" t="s">
-        <v>273</v>
       </c>
       <c r="F116" t="s">
         <v>6</v>
@@ -3709,19 +3709,19 @@
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B117" t="s">
+        <v>271</v>
+      </c>
+      <c r="C117" t="s">
+        <v>27</v>
+      </c>
+      <c r="D117" t="s">
+        <v>278</v>
+      </c>
+      <c r="E117" t="s">
         <v>272</v>
-      </c>
-      <c r="C117" t="s">
-        <v>28</v>
-      </c>
-      <c r="D117" t="s">
-        <v>279</v>
-      </c>
-      <c r="E117" t="s">
-        <v>273</v>
       </c>
       <c r="F117" t="s">
         <v>6</v>
@@ -3729,19 +3729,19 @@
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B118" t="s">
+        <v>280</v>
+      </c>
+      <c r="C118" t="s">
+        <v>296</v>
+      </c>
+      <c r="D118" t="s">
         <v>281</v>
       </c>
-      <c r="C118" t="s">
-        <v>297</v>
-      </c>
-      <c r="D118" t="s">
-        <v>282</v>
-      </c>
       <c r="E118" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F118" t="s">
         <v>6</v>
@@ -3749,19 +3749,19 @@
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B119" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C119" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="D119" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="E119" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F119" t="s">
         <v>6</v>
@@ -3769,19 +3769,19 @@
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
+        <v>284</v>
+      </c>
+      <c r="B120" t="s">
+        <v>280</v>
+      </c>
+      <c r="C120" t="s">
+        <v>296</v>
+      </c>
+      <c r="D120" t="s">
         <v>285</v>
       </c>
-      <c r="B120" t="s">
-        <v>281</v>
-      </c>
-      <c r="C120" t="s">
-        <v>297</v>
-      </c>
-      <c r="D120" t="s">
-        <v>286</v>
-      </c>
       <c r="E120" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F120" t="s">
         <v>6</v>
@@ -3789,19 +3789,19 @@
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B121" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C121" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="D121" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="E121" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F121" t="s">
         <v>6</v>
@@ -3809,19 +3809,19 @@
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B122" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C122" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="D122" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="E122" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F122" t="s">
         <v>6</v>
@@ -3829,19 +3829,19 @@
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
+        <v>290</v>
+      </c>
+      <c r="B123" t="s">
+        <v>280</v>
+      </c>
+      <c r="C123" t="s">
+        <v>296</v>
+      </c>
+      <c r="D123" t="s">
         <v>291</v>
       </c>
-      <c r="B123" t="s">
-        <v>281</v>
-      </c>
-      <c r="C123" t="s">
-        <v>297</v>
-      </c>
-      <c r="D123" t="s">
-        <v>292</v>
-      </c>
       <c r="E123" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F123" t="s">
         <v>6</v>
@@ -3849,19 +3849,19 @@
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
+        <v>292</v>
+      </c>
+      <c r="B124" t="s">
+        <v>280</v>
+      </c>
+      <c r="C124" t="s">
+        <v>296</v>
+      </c>
+      <c r="D124" t="s">
         <v>293</v>
       </c>
-      <c r="B124" t="s">
-        <v>281</v>
-      </c>
-      <c r="C124" t="s">
-        <v>297</v>
-      </c>
-      <c r="D124" t="s">
+      <c r="E124" t="s">
         <v>294</v>
-      </c>
-      <c r="E124" t="s">
-        <v>295</v>
       </c>
       <c r="F124" t="s">
         <v>6</v>
@@ -3869,162 +3869,162 @@
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
+        <v>302</v>
+      </c>
+      <c r="B125" t="s">
         <v>303</v>
-      </c>
-      <c r="B125" t="s">
-        <v>304</v>
       </c>
       <c r="C125" t="s">
         <v>7</v>
       </c>
       <c r="D125" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="E125" t="s">
+        <v>304</v>
+      </c>
+      <c r="F125" t="s">
         <v>305</v>
-      </c>
-      <c r="F125" t="s">
-        <v>306</v>
       </c>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B126" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C126" t="s">
         <v>7</v>
       </c>
       <c r="D126" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="E126" t="s">
+        <v>304</v>
+      </c>
+      <c r="F126" t="s">
         <v>305</v>
-      </c>
-      <c r="F126" t="s">
-        <v>306</v>
       </c>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="B127" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C127" t="s">
         <v>7</v>
       </c>
       <c r="D127" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="E127" t="s">
+        <v>304</v>
+      </c>
+      <c r="F127" t="s">
         <v>305</v>
-      </c>
-      <c r="F127" t="s">
-        <v>306</v>
       </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="B128" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C128" t="s">
         <v>7</v>
       </c>
       <c r="D128" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E128" t="s">
+        <v>304</v>
+      </c>
+      <c r="F128" t="s">
         <v>305</v>
-      </c>
-      <c r="F128" t="s">
-        <v>306</v>
       </c>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="B129" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C129" t="s">
         <v>7</v>
       </c>
       <c r="D129" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="E129" t="s">
+        <v>304</v>
+      </c>
+      <c r="F129" t="s">
         <v>305</v>
-      </c>
-      <c r="F129" t="s">
-        <v>306</v>
       </c>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B130" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C130" t="s">
         <v>7</v>
       </c>
       <c r="D130" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="E130" t="s">
+        <v>304</v>
+      </c>
+      <c r="F130" t="s">
         <v>305</v>
-      </c>
-      <c r="F130" t="s">
-        <v>306</v>
       </c>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B131" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C131" t="s">
         <v>7</v>
       </c>
       <c r="D131" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="E131" t="s">
+        <v>304</v>
+      </c>
+      <c r="F131" t="s">
         <v>305</v>
-      </c>
-      <c r="F131" t="s">
-        <v>306</v>
       </c>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B132" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C132" t="s">
         <v>7</v>
       </c>
       <c r="D132" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="E132" t="s">
+        <v>304</v>
+      </c>
+      <c r="F132" t="s">
         <v>305</v>
-      </c>
-      <c r="F132" t="s">
-        <v>306</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Katalog guncellendi - 19.06.2026 17:32:09,18
</commit_message>
<xml_diff>
--- a/urunler.xlsx
+++ b/urunler.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/49dd5535ee0ab452/Desktop/CEREN-PC/SIVAL_GIYIM_KATALOG/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/49dd5535ee0ab452/Desktop/YEMEK LİSTELERİ/yemek/CEREN-PC/SIVAL_GIYIM_KATALOG/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="200" documentId="13_ncr:1_{CCE8B614-DB69-4334-AC06-D714AC841E42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6CCB6A72-3E60-4DF3-AF20-E3F47A40E665}"/>
+  <xr:revisionPtr revIDLastSave="214" documentId="13_ncr:1_{CCE8B614-DB69-4334-AC06-D714AC841E42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{50ABA224-DFB3-445E-B080-66A8B0F3AEEA}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -61,9 +61,6 @@
     <t>Baggy Siyah</t>
   </si>
   <si>
-    <t>300 TL</t>
-  </si>
-  <si>
     <t>BAG6.jpg</t>
   </si>
   <si>
@@ -983,6 +980,9 @@
   </si>
   <si>
     <t>350TL</t>
+  </si>
+  <si>
+    <t>350 Tl</t>
   </si>
 </sst>
 </file>
@@ -1412,7 +1412,7 @@
         <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C2" t="s">
         <v>7</v>
@@ -1421,7 +1421,7 @@
         <v>8</v>
       </c>
       <c r="E2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F2" t="s">
         <v>6</v>
@@ -1432,7 +1432,7 @@
         <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C3" t="s">
         <v>7</v>
@@ -1441,7 +1441,7 @@
         <v>9</v>
       </c>
       <c r="E3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F3" t="s">
         <v>6</v>
@@ -1452,36 +1452,36 @@
         <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C4" t="s">
         <v>7</v>
       </c>
       <c r="D4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F4" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B5" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C5" t="s">
         <v>7</v>
       </c>
       <c r="D5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F5" t="s">
         <v>6</v>
@@ -1489,19 +1489,19 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C6" t="s">
         <v>7</v>
       </c>
       <c r="D6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F6" t="s">
         <v>6</v>
@@ -1509,19 +1509,19 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B7" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C7" t="s">
         <v>7</v>
       </c>
       <c r="D7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E7" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F7" t="s">
         <v>6</v>
@@ -1529,39 +1529,39 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B8" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C8" t="s">
         <v>7</v>
       </c>
       <c r="D8" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B9" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C9" t="s">
         <v>7</v>
       </c>
       <c r="D9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F9" t="s">
         <v>6</v>
@@ -1569,19 +1569,19 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B10" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C10" t="s">
         <v>7</v>
       </c>
       <c r="D10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F10" t="s">
         <v>6</v>
@@ -1589,19 +1589,19 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B11" t="s">
-        <v>13</v>
+        <v>320</v>
       </c>
       <c r="C11" t="s">
+        <v>26</v>
+      </c>
+      <c r="D11" t="s">
         <v>27</v>
       </c>
-      <c r="D11" t="s">
-        <v>28</v>
-      </c>
       <c r="E11" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F11" t="s">
         <v>6</v>
@@ -1609,39 +1609,39 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>29</v>
+      </c>
+      <c r="B12" t="s">
+        <v>320</v>
+      </c>
+      <c r="C12" t="s">
+        <v>26</v>
+      </c>
+      <c r="D12" t="s">
         <v>30</v>
       </c>
-      <c r="B12" t="s">
-        <v>13</v>
-      </c>
-      <c r="C12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D12" t="s">
-        <v>31</v>
-      </c>
       <c r="E12" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F12" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>32</v>
+      </c>
+      <c r="B13" t="s">
+        <v>320</v>
+      </c>
+      <c r="C13" t="s">
+        <v>26</v>
+      </c>
+      <c r="D13" t="s">
         <v>33</v>
       </c>
-      <c r="B13" t="s">
-        <v>13</v>
-      </c>
-      <c r="C13" t="s">
-        <v>27</v>
-      </c>
-      <c r="D13" t="s">
-        <v>34</v>
-      </c>
       <c r="E13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F13" t="s">
         <v>6</v>
@@ -1649,19 +1649,19 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>34</v>
+      </c>
+      <c r="B14" t="s">
+        <v>320</v>
+      </c>
+      <c r="C14" t="s">
+        <v>26</v>
+      </c>
+      <c r="D14" t="s">
         <v>35</v>
       </c>
-      <c r="B14" t="s">
-        <v>13</v>
-      </c>
-      <c r="C14" t="s">
-        <v>27</v>
-      </c>
-      <c r="D14" t="s">
-        <v>36</v>
-      </c>
       <c r="E14" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F14" t="s">
         <v>6</v>
@@ -1669,19 +1669,19 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>36</v>
+      </c>
+      <c r="B15" t="s">
+        <v>320</v>
+      </c>
+      <c r="C15" t="s">
+        <v>26</v>
+      </c>
+      <c r="D15" t="s">
         <v>37</v>
       </c>
-      <c r="B15" t="s">
-        <v>13</v>
-      </c>
-      <c r="C15" t="s">
-        <v>27</v>
-      </c>
-      <c r="D15" t="s">
-        <v>38</v>
-      </c>
       <c r="E15" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F15" t="s">
         <v>6</v>
@@ -1689,19 +1689,19 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>38</v>
+      </c>
+      <c r="B16" t="s">
+        <v>320</v>
+      </c>
+      <c r="C16" t="s">
+        <v>26</v>
+      </c>
+      <c r="D16" t="s">
         <v>39</v>
       </c>
-      <c r="B16" t="s">
-        <v>13</v>
-      </c>
-      <c r="C16" t="s">
-        <v>27</v>
-      </c>
-      <c r="D16" t="s">
-        <v>40</v>
-      </c>
       <c r="E16" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F16" t="s">
         <v>6</v>
@@ -1709,19 +1709,19 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>40</v>
+      </c>
+      <c r="B17" t="s">
+        <v>320</v>
+      </c>
+      <c r="C17" t="s">
+        <v>26</v>
+      </c>
+      <c r="D17" t="s">
         <v>41</v>
       </c>
-      <c r="B17" t="s">
-        <v>13</v>
-      </c>
-      <c r="C17" t="s">
-        <v>27</v>
-      </c>
-      <c r="D17" t="s">
-        <v>42</v>
-      </c>
       <c r="E17" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F17" t="s">
         <v>6</v>
@@ -1729,19 +1729,19 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>42</v>
+      </c>
+      <c r="B18" t="s">
+        <v>320</v>
+      </c>
+      <c r="C18" t="s">
+        <v>26</v>
+      </c>
+      <c r="D18" t="s">
         <v>43</v>
       </c>
-      <c r="B18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C18" t="s">
-        <v>27</v>
-      </c>
-      <c r="D18" t="s">
-        <v>44</v>
-      </c>
       <c r="E18" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F18" t="s">
         <v>6</v>
@@ -1749,19 +1749,19 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>44</v>
+      </c>
+      <c r="B19" t="s">
+        <v>320</v>
+      </c>
+      <c r="C19" t="s">
+        <v>26</v>
+      </c>
+      <c r="D19" t="s">
         <v>45</v>
       </c>
-      <c r="B19" t="s">
-        <v>13</v>
-      </c>
-      <c r="C19" t="s">
-        <v>27</v>
-      </c>
-      <c r="D19" t="s">
-        <v>46</v>
-      </c>
       <c r="E19" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F19" t="s">
         <v>6</v>
@@ -1769,19 +1769,19 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>46</v>
+      </c>
+      <c r="B20" t="s">
+        <v>320</v>
+      </c>
+      <c r="C20" t="s">
+        <v>26</v>
+      </c>
+      <c r="D20" t="s">
         <v>47</v>
       </c>
-      <c r="B20" t="s">
-        <v>13</v>
-      </c>
-      <c r="C20" t="s">
-        <v>27</v>
-      </c>
-      <c r="D20" t="s">
-        <v>48</v>
-      </c>
       <c r="E20" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F20" t="s">
         <v>6</v>
@@ -1789,19 +1789,19 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>48</v>
+      </c>
+      <c r="B21" t="s">
+        <v>320</v>
+      </c>
+      <c r="C21" t="s">
+        <v>26</v>
+      </c>
+      <c r="D21" t="s">
         <v>49</v>
       </c>
-      <c r="B21" t="s">
-        <v>13</v>
-      </c>
-      <c r="C21" t="s">
-        <v>27</v>
-      </c>
-      <c r="D21" t="s">
-        <v>50</v>
-      </c>
       <c r="E21" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F21" t="s">
         <v>6</v>
@@ -1809,19 +1809,19 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B22" t="s">
-        <v>13</v>
+        <v>320</v>
       </c>
       <c r="C22" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D22" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E22" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F22" t="s">
         <v>6</v>
@@ -1829,19 +1829,19 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B23" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C23" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D23" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E23" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F23" t="s">
         <v>6</v>
@@ -1849,19 +1849,19 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>54</v>
+      </c>
+      <c r="B24" t="s">
+        <v>125</v>
+      </c>
+      <c r="C24" t="s">
+        <v>26</v>
+      </c>
+      <c r="D24" t="s">
         <v>55</v>
       </c>
-      <c r="B24" t="s">
-        <v>126</v>
-      </c>
-      <c r="C24" t="s">
-        <v>27</v>
-      </c>
-      <c r="D24" t="s">
-        <v>56</v>
-      </c>
       <c r="E24" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F24" t="s">
         <v>6</v>
@@ -1869,19 +1869,19 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>56</v>
+      </c>
+      <c r="B25" t="s">
+        <v>125</v>
+      </c>
+      <c r="C25" t="s">
+        <v>26</v>
+      </c>
+      <c r="D25" t="s">
         <v>57</v>
       </c>
-      <c r="B25" t="s">
-        <v>126</v>
-      </c>
-      <c r="C25" t="s">
-        <v>27</v>
-      </c>
-      <c r="D25" t="s">
-        <v>58</v>
-      </c>
       <c r="E25" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F25" t="s">
         <v>6</v>
@@ -1889,19 +1889,19 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B26" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C26" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D26" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F26" t="s">
         <v>6</v>
@@ -1909,19 +1909,19 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>60</v>
+      </c>
+      <c r="B27" t="s">
+        <v>126</v>
+      </c>
+      <c r="C27" t="s">
+        <v>26</v>
+      </c>
+      <c r="D27" t="s">
         <v>61</v>
       </c>
-      <c r="B27" t="s">
-        <v>127</v>
-      </c>
-      <c r="C27" t="s">
-        <v>27</v>
-      </c>
-      <c r="D27" t="s">
-        <v>62</v>
-      </c>
       <c r="E27" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F27" t="s">
         <v>6</v>
@@ -1929,19 +1929,19 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
+        <v>62</v>
+      </c>
+      <c r="B28" t="s">
+        <v>126</v>
+      </c>
+      <c r="C28" t="s">
+        <v>26</v>
+      </c>
+      <c r="D28" t="s">
         <v>63</v>
       </c>
-      <c r="B28" t="s">
-        <v>127</v>
-      </c>
-      <c r="C28" t="s">
-        <v>27</v>
-      </c>
-      <c r="D28" t="s">
-        <v>64</v>
-      </c>
       <c r="E28" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F28" t="s">
         <v>6</v>
@@ -1949,19 +1949,19 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>64</v>
+      </c>
+      <c r="B29" t="s">
+        <v>126</v>
+      </c>
+      <c r="C29" t="s">
+        <v>26</v>
+      </c>
+      <c r="D29" t="s">
         <v>65</v>
       </c>
-      <c r="B29" t="s">
-        <v>127</v>
-      </c>
-      <c r="C29" t="s">
-        <v>27</v>
-      </c>
-      <c r="D29" t="s">
-        <v>66</v>
-      </c>
       <c r="E29" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F29" t="s">
         <v>6</v>
@@ -1969,19 +1969,19 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B30" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C30" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D30" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F30" t="s">
         <v>6</v>
@@ -1989,19 +1989,19 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B31" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C31" t="s">
         <v>7</v>
       </c>
       <c r="D31" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F31" t="s">
         <v>6</v>
@@ -2009,19 +2009,19 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B32" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C32" t="s">
         <v>7</v>
       </c>
       <c r="D32" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F32" t="s">
         <v>6</v>
@@ -2029,19 +2029,19 @@
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B33" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C33" t="s">
         <v>7</v>
       </c>
       <c r="D33" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F33" t="s">
         <v>6</v>
@@ -2049,19 +2049,19 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B34" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C34" t="s">
         <v>7</v>
       </c>
       <c r="D34" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F34" t="s">
         <v>6</v>
@@ -2069,19 +2069,19 @@
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B35" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C35" t="s">
         <v>7</v>
       </c>
       <c r="D35" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F35" t="s">
         <v>6</v>
@@ -2089,19 +2089,19 @@
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B36" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C36" t="s">
         <v>7</v>
       </c>
       <c r="D36" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F36" t="s">
         <v>6</v>
@@ -2109,19 +2109,19 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B37" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C37" t="s">
         <v>7</v>
       </c>
       <c r="D37" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F37" t="s">
         <v>6</v>
@@ -2129,19 +2129,19 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B38" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C38" t="s">
         <v>7</v>
       </c>
       <c r="D38" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F38" t="s">
         <v>6</v>
@@ -2149,19 +2149,19 @@
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B39" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C39" t="s">
         <v>7</v>
       </c>
       <c r="D39" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F39" t="s">
         <v>6</v>
@@ -2169,19 +2169,19 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B40" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C40" t="s">
         <v>7</v>
       </c>
       <c r="D40" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F40" t="s">
         <v>6</v>
@@ -2189,19 +2189,19 @@
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B41" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C41" t="s">
         <v>7</v>
       </c>
       <c r="D41" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F41" t="s">
         <v>6</v>
@@ -2209,19 +2209,19 @@
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B42" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C42" t="s">
         <v>7</v>
       </c>
       <c r="D42" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F42" t="s">
         <v>6</v>
@@ -2229,19 +2229,19 @@
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B43" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C43" t="s">
         <v>7</v>
       </c>
       <c r="D43" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F43" t="s">
         <v>6</v>
@@ -2249,19 +2249,19 @@
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B44" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C44" t="s">
         <v>7</v>
       </c>
       <c r="D44" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F44" t="s">
         <v>6</v>
@@ -2269,19 +2269,19 @@
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B45" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C45" t="s">
         <v>7</v>
       </c>
       <c r="D45" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F45" t="s">
         <v>6</v>
@@ -2289,19 +2289,19 @@
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B46" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C46" t="s">
         <v>7</v>
       </c>
       <c r="D46" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F46" t="s">
         <v>6</v>
@@ -2309,19 +2309,19 @@
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B47" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C47" t="s">
         <v>7</v>
       </c>
       <c r="D47" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F47" t="s">
         <v>6</v>
@@ -2329,19 +2329,19 @@
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B48" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C48" t="s">
         <v>7</v>
       </c>
       <c r="D48" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F48" t="s">
         <v>6</v>
@@ -2349,19 +2349,19 @@
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B49" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C49" t="s">
         <v>7</v>
       </c>
       <c r="D49" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F49" t="s">
         <v>6</v>
@@ -2369,19 +2369,19 @@
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B50" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C50" t="s">
         <v>7</v>
       </c>
       <c r="D50" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F50" t="s">
         <v>6</v>
@@ -2389,19 +2389,19 @@
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C51" t="s">
         <v>7</v>
       </c>
       <c r="D51" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F51" t="s">
         <v>6</v>
@@ -2409,19 +2409,19 @@
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B52" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C52" t="s">
         <v>7</v>
       </c>
       <c r="D52" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F52" t="s">
         <v>6</v>
@@ -2429,19 +2429,19 @@
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
+        <v>111</v>
+      </c>
+      <c r="B53" t="s">
+        <v>128</v>
+      </c>
+      <c r="C53" t="s">
         <v>112</v>
       </c>
-      <c r="B53" t="s">
-        <v>129</v>
-      </c>
-      <c r="C53" t="s">
+      <c r="D53" t="s">
+        <v>136</v>
+      </c>
+      <c r="E53" t="s">
         <v>113</v>
-      </c>
-      <c r="D53" t="s">
-        <v>137</v>
-      </c>
-      <c r="E53" t="s">
-        <v>114</v>
       </c>
       <c r="F53" t="s">
         <v>6</v>
@@ -2449,19 +2449,19 @@
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
+        <v>114</v>
+      </c>
+      <c r="B54" t="s">
+        <v>128</v>
+      </c>
+      <c r="C54" t="s">
+        <v>112</v>
+      </c>
+      <c r="D54" t="s">
         <v>115</v>
       </c>
-      <c r="B54" t="s">
-        <v>129</v>
-      </c>
-      <c r="C54" t="s">
+      <c r="E54" t="s">
         <v>113</v>
-      </c>
-      <c r="D54" t="s">
-        <v>116</v>
-      </c>
-      <c r="E54" t="s">
-        <v>114</v>
       </c>
       <c r="F54" t="s">
         <v>6</v>
@@ -2469,19 +2469,19 @@
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
+        <v>116</v>
+      </c>
+      <c r="B55" t="s">
+        <v>128</v>
+      </c>
+      <c r="C55" t="s">
+        <v>112</v>
+      </c>
+      <c r="D55" t="s">
         <v>117</v>
       </c>
-      <c r="B55" t="s">
-        <v>129</v>
-      </c>
-      <c r="C55" t="s">
+      <c r="E55" t="s">
         <v>113</v>
-      </c>
-      <c r="D55" t="s">
-        <v>118</v>
-      </c>
-      <c r="E55" t="s">
-        <v>114</v>
       </c>
       <c r="F55" t="s">
         <v>6</v>
@@ -2489,19 +2489,19 @@
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B56" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C56" t="s">
         <v>7</v>
       </c>
       <c r="D56" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E56" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F56" t="s">
         <v>6</v>
@@ -2509,19 +2509,19 @@
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B57" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C57" t="s">
         <v>7</v>
       </c>
       <c r="D57" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E57" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F57" t="s">
         <v>6</v>
@@ -2529,219 +2529,219 @@
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
+        <v>137</v>
+      </c>
+      <c r="B58" t="s">
         <v>138</v>
       </c>
-      <c r="B58" t="s">
+      <c r="C58" t="s">
+        <v>112</v>
+      </c>
+      <c r="D58" t="s">
+        <v>140</v>
+      </c>
+      <c r="E58" t="s">
         <v>139</v>
       </c>
-      <c r="C58" t="s">
-        <v>113</v>
-      </c>
-      <c r="D58" t="s">
-        <v>141</v>
-      </c>
-      <c r="E58" t="s">
-        <v>140</v>
-      </c>
       <c r="F58" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B59" t="s">
+        <v>138</v>
+      </c>
+      <c r="C59" t="s">
+        <v>112</v>
+      </c>
+      <c r="D59" t="s">
+        <v>141</v>
+      </c>
+      <c r="E59" t="s">
         <v>139</v>
       </c>
-      <c r="C59" t="s">
-        <v>113</v>
-      </c>
-      <c r="D59" t="s">
-        <v>142</v>
-      </c>
-      <c r="E59" t="s">
-        <v>140</v>
-      </c>
       <c r="F59" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B60" t="s">
+        <v>138</v>
+      </c>
+      <c r="C60" t="s">
+        <v>112</v>
+      </c>
+      <c r="D60" t="s">
+        <v>143</v>
+      </c>
+      <c r="E60" t="s">
         <v>139</v>
       </c>
-      <c r="C60" t="s">
-        <v>113</v>
-      </c>
-      <c r="D60" t="s">
-        <v>144</v>
-      </c>
-      <c r="E60" t="s">
-        <v>140</v>
-      </c>
       <c r="F60" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B61" t="s">
+        <v>138</v>
+      </c>
+      <c r="C61" t="s">
+        <v>112</v>
+      </c>
+      <c r="D61" t="s">
+        <v>145</v>
+      </c>
+      <c r="E61" t="s">
         <v>139</v>
       </c>
-      <c r="C61" t="s">
-        <v>113</v>
-      </c>
-      <c r="D61" t="s">
-        <v>146</v>
-      </c>
-      <c r="E61" t="s">
-        <v>140</v>
-      </c>
       <c r="F61" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B62" t="s">
+        <v>138</v>
+      </c>
+      <c r="C62" t="s">
+        <v>112</v>
+      </c>
+      <c r="D62" t="s">
+        <v>147</v>
+      </c>
+      <c r="E62" t="s">
         <v>139</v>
       </c>
-      <c r="C62" t="s">
-        <v>113</v>
-      </c>
-      <c r="D62" t="s">
-        <v>148</v>
-      </c>
-      <c r="E62" t="s">
-        <v>140</v>
-      </c>
       <c r="F62" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B63" t="s">
+        <v>138</v>
+      </c>
+      <c r="C63" t="s">
+        <v>112</v>
+      </c>
+      <c r="D63" t="s">
+        <v>149</v>
+      </c>
+      <c r="E63" t="s">
         <v>139</v>
       </c>
-      <c r="C63" t="s">
-        <v>113</v>
-      </c>
-      <c r="D63" t="s">
-        <v>150</v>
-      </c>
-      <c r="E63" t="s">
-        <v>140</v>
-      </c>
       <c r="F63" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
+        <v>151</v>
+      </c>
+      <c r="B64" t="s">
+        <v>153</v>
+      </c>
+      <c r="C64" t="s">
+        <v>112</v>
+      </c>
+      <c r="D64" t="s">
         <v>152</v>
       </c>
-      <c r="B64" t="s">
-        <v>154</v>
-      </c>
-      <c r="C64" t="s">
-        <v>113</v>
-      </c>
-      <c r="D64" t="s">
-        <v>153</v>
-      </c>
       <c r="E64" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F64" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B65" s="4" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C65" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D65" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E65" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F65" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B66" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C66" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D66" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E66" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F66" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B67" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C67" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D67" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="E67" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F67" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
+        <v>159</v>
+      </c>
+      <c r="B68" t="s">
         <v>160</v>
       </c>
-      <c r="B68" t="s">
-        <v>161</v>
-      </c>
       <c r="C68" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D68" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="E68" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F68" t="s">
         <v>6</v>
@@ -2749,119 +2749,119 @@
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B69" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C69" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D69" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E69" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F69" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
+        <v>165</v>
+      </c>
+      <c r="B70" t="s">
         <v>166</v>
       </c>
-      <c r="B70" t="s">
-        <v>167</v>
-      </c>
       <c r="C70" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D70" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E70" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F70" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B71" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C71" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D71" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E71" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F71" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B72" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C72" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D72" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E72" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F72" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
+        <v>172</v>
+      </c>
+      <c r="B73" t="s">
         <v>173</v>
       </c>
-      <c r="B73" t="s">
-        <v>174</v>
-      </c>
       <c r="C73" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D73" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E73" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F73" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B74" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C74" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D74" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="E74" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F74" t="s">
         <v>6</v>
@@ -2869,19 +2869,19 @@
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B75" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C75" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D75" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E75" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F75" t="s">
         <v>6</v>
@@ -2889,19 +2889,19 @@
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B76" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C76" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D76" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E76" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F76" t="s">
         <v>6</v>
@@ -2909,19 +2909,19 @@
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B77" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C77" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D77" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E77" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F77" t="s">
         <v>6</v>
@@ -2929,19 +2929,19 @@
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B78" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C78" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D78" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E78" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F78" t="s">
         <v>6</v>
@@ -2949,19 +2949,19 @@
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
+        <v>189</v>
+      </c>
+      <c r="B79" t="s">
+        <v>125</v>
+      </c>
+      <c r="C79" t="s">
         <v>190</v>
       </c>
-      <c r="B79" t="s">
-        <v>126</v>
-      </c>
-      <c r="C79" t="s">
-        <v>191</v>
-      </c>
       <c r="D79" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="E79" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F79" t="s">
         <v>6</v>
@@ -2969,19 +2969,19 @@
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
+        <v>191</v>
+      </c>
+      <c r="B80" t="s">
         <v>192</v>
       </c>
-      <c r="B80" t="s">
+      <c r="C80" t="s">
+        <v>190</v>
+      </c>
+      <c r="D80" t="s">
         <v>193</v>
       </c>
-      <c r="C80" t="s">
-        <v>191</v>
-      </c>
-      <c r="D80" t="s">
-        <v>194</v>
-      </c>
       <c r="E80" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F80" t="s">
         <v>6</v>
@@ -2989,19 +2989,19 @@
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B81" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C81" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D81" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E81" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F81" t="s">
         <v>6</v>
@@ -3009,19 +3009,19 @@
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
+        <v>196</v>
+      </c>
+      <c r="B82" t="s">
+        <v>192</v>
+      </c>
+      <c r="C82" t="s">
+        <v>190</v>
+      </c>
+      <c r="D82" t="s">
         <v>197</v>
       </c>
-      <c r="B82" t="s">
-        <v>193</v>
-      </c>
-      <c r="C82" t="s">
-        <v>191</v>
-      </c>
-      <c r="D82" t="s">
-        <v>198</v>
-      </c>
       <c r="E82" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F82" t="s">
         <v>6</v>
@@ -3029,19 +3029,19 @@
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
+        <v>198</v>
+      </c>
+      <c r="B83" t="s">
+        <v>192</v>
+      </c>
+      <c r="C83" t="s">
+        <v>190</v>
+      </c>
+      <c r="D83" t="s">
         <v>199</v>
       </c>
-      <c r="B83" t="s">
-        <v>193</v>
-      </c>
-      <c r="C83" t="s">
-        <v>191</v>
-      </c>
-      <c r="D83" t="s">
-        <v>200</v>
-      </c>
       <c r="E83" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F83" t="s">
         <v>6</v>
@@ -3049,19 +3049,19 @@
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B84" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C84" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D84" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E84" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F84" t="s">
         <v>6</v>
@@ -3069,19 +3069,19 @@
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B85" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C85" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D85" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E85" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F85" t="s">
         <v>6</v>
@@ -3089,19 +3089,19 @@
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B86" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C86" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D86" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="E86" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F86" t="s">
         <v>6</v>
@@ -3109,19 +3109,19 @@
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
+        <v>208</v>
+      </c>
+      <c r="B87" t="s">
+        <v>192</v>
+      </c>
+      <c r="C87" t="s">
+        <v>190</v>
+      </c>
+      <c r="D87" t="s">
+        <v>204</v>
+      </c>
+      <c r="E87" t="s">
         <v>209</v>
-      </c>
-      <c r="B87" t="s">
-        <v>193</v>
-      </c>
-      <c r="C87" t="s">
-        <v>191</v>
-      </c>
-      <c r="D87" t="s">
-        <v>205</v>
-      </c>
-      <c r="E87" t="s">
-        <v>210</v>
       </c>
       <c r="F87" t="s">
         <v>6</v>
@@ -3129,19 +3129,19 @@
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B88" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C88" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D88" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E88" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F88" t="s">
         <v>6</v>
@@ -3149,19 +3149,19 @@
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
+        <v>210</v>
+      </c>
+      <c r="B89" t="s">
         <v>211</v>
       </c>
-      <c r="B89" t="s">
+      <c r="C89" t="s">
         <v>212</v>
       </c>
-      <c r="C89" t="s">
+      <c r="D89" t="s">
         <v>213</v>
       </c>
-      <c r="D89" t="s">
+      <c r="E89" t="s">
         <v>214</v>
-      </c>
-      <c r="E89" t="s">
-        <v>215</v>
       </c>
       <c r="F89" t="s">
         <v>6</v>
@@ -3169,19 +3169,19 @@
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B90" t="s">
+        <v>211</v>
+      </c>
+      <c r="C90" t="s">
         <v>212</v>
       </c>
-      <c r="C90" t="s">
-        <v>213</v>
-      </c>
       <c r="D90" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="E90" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F90" t="s">
         <v>6</v>
@@ -3189,19 +3189,19 @@
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B91" t="s">
+        <v>211</v>
+      </c>
+      <c r="C91" t="s">
         <v>212</v>
       </c>
-      <c r="C91" t="s">
-        <v>213</v>
-      </c>
       <c r="D91" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="E91" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F91" t="s">
         <v>6</v>
@@ -3209,19 +3209,19 @@
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B92" t="s">
+        <v>211</v>
+      </c>
+      <c r="C92" t="s">
         <v>212</v>
       </c>
-      <c r="C92" t="s">
-        <v>213</v>
-      </c>
       <c r="D92" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="E92" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F92" t="s">
         <v>6</v>
@@ -3229,19 +3229,19 @@
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B93" t="s">
+        <v>211</v>
+      </c>
+      <c r="C93" t="s">
         <v>212</v>
       </c>
-      <c r="C93" t="s">
-        <v>213</v>
-      </c>
       <c r="D93" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E93" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F93" t="s">
         <v>6</v>
@@ -3249,19 +3249,19 @@
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B94" t="s">
+        <v>211</v>
+      </c>
+      <c r="C94" t="s">
         <v>212</v>
       </c>
-      <c r="C94" t="s">
-        <v>213</v>
-      </c>
       <c r="D94" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E94" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F94" t="s">
         <v>6</v>
@@ -3269,19 +3269,19 @@
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B95" t="s">
+        <v>211</v>
+      </c>
+      <c r="C95" t="s">
         <v>212</v>
       </c>
-      <c r="C95" t="s">
-        <v>213</v>
-      </c>
       <c r="D95" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E95" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F95" t="s">
         <v>6</v>
@@ -3289,19 +3289,19 @@
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B96" t="s">
+        <v>211</v>
+      </c>
+      <c r="C96" t="s">
         <v>212</v>
       </c>
-      <c r="C96" t="s">
-        <v>213</v>
-      </c>
       <c r="D96" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="E96" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F96" t="s">
         <v>6</v>
@@ -3309,19 +3309,19 @@
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B97" t="s">
+        <v>211</v>
+      </c>
+      <c r="C97" t="s">
         <v>212</v>
       </c>
-      <c r="C97" t="s">
-        <v>213</v>
-      </c>
       <c r="D97" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E97" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F97" t="s">
         <v>6</v>
@@ -3329,19 +3329,19 @@
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
+        <v>231</v>
+      </c>
+      <c r="B98" t="s">
+        <v>125</v>
+      </c>
+      <c r="C98" t="s">
+        <v>212</v>
+      </c>
+      <c r="D98" t="s">
         <v>232</v>
       </c>
-      <c r="B98" t="s">
-        <v>126</v>
-      </c>
-      <c r="C98" t="s">
-        <v>213</v>
-      </c>
-      <c r="D98" t="s">
-        <v>233</v>
-      </c>
       <c r="E98" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F98" t="s">
         <v>6</v>
@@ -3349,19 +3349,19 @@
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B99" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C99" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D99" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E99" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F99" t="s">
         <v>6</v>
@@ -3369,19 +3369,19 @@
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B100" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C100" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D100" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E100" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F100" t="s">
         <v>6</v>
@@ -3389,19 +3389,19 @@
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
+        <v>235</v>
+      </c>
+      <c r="B101" t="s">
         <v>236</v>
       </c>
-      <c r="B101" t="s">
+      <c r="C101" t="s">
+        <v>190</v>
+      </c>
+      <c r="D101" t="s">
         <v>237</v>
       </c>
-      <c r="C101" t="s">
-        <v>191</v>
-      </c>
-      <c r="D101" t="s">
-        <v>238</v>
-      </c>
       <c r="E101" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F101" t="s">
         <v>6</v>
@@ -3409,19 +3409,19 @@
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B102" t="s">
+        <v>238</v>
+      </c>
+      <c r="C102" t="s">
+        <v>190</v>
+      </c>
+      <c r="D102" t="s">
         <v>239</v>
       </c>
-      <c r="C102" t="s">
-        <v>191</v>
-      </c>
-      <c r="D102" t="s">
-        <v>240</v>
-      </c>
       <c r="E102" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F102" t="s">
         <v>6</v>
@@ -3429,19 +3429,19 @@
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B103" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C103" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D103" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E103" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F103" t="s">
         <v>6</v>
@@ -3449,19 +3449,19 @@
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B104" t="s">
+        <v>246</v>
+      </c>
+      <c r="C104" t="s">
+        <v>190</v>
+      </c>
+      <c r="D104" t="s">
         <v>247</v>
       </c>
-      <c r="C104" t="s">
-        <v>191</v>
-      </c>
-      <c r="D104" t="s">
-        <v>248</v>
-      </c>
       <c r="E104" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F104" t="s">
         <v>6</v>
@@ -3469,19 +3469,19 @@
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
+        <v>245</v>
+      </c>
+      <c r="B105" t="s">
         <v>246</v>
       </c>
-      <c r="B105" t="s">
-        <v>247</v>
-      </c>
       <c r="C105" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D105" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="E105" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F105" t="s">
         <v>6</v>
@@ -3489,19 +3489,19 @@
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B106" t="s">
+        <v>249</v>
+      </c>
+      <c r="C106" t="s">
         <v>250</v>
       </c>
-      <c r="C106" t="s">
+      <c r="D106" t="s">
         <v>251</v>
       </c>
-      <c r="D106" t="s">
-        <v>252</v>
-      </c>
       <c r="E106" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="F106" t="s">
         <v>6</v>
@@ -3509,19 +3509,19 @@
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B107" t="s">
+        <v>249</v>
+      </c>
+      <c r="C107" t="s">
         <v>250</v>
       </c>
-      <c r="C107" t="s">
-        <v>251</v>
-      </c>
       <c r="D107" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="E107" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="F107" t="s">
         <v>6</v>
@@ -3529,19 +3529,19 @@
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B108" t="s">
+        <v>249</v>
+      </c>
+      <c r="C108" t="s">
         <v>250</v>
       </c>
-      <c r="C108" t="s">
-        <v>251</v>
-      </c>
       <c r="D108" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E108" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="F108" t="s">
         <v>6</v>
@@ -3549,19 +3549,19 @@
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
+        <v>258</v>
+      </c>
+      <c r="B109" t="s">
+        <v>249</v>
+      </c>
+      <c r="C109" t="s">
+        <v>250</v>
+      </c>
+      <c r="D109" t="s">
+        <v>257</v>
+      </c>
+      <c r="E109" t="s">
         <v>259</v>
-      </c>
-      <c r="B109" t="s">
-        <v>250</v>
-      </c>
-      <c r="C109" t="s">
-        <v>251</v>
-      </c>
-      <c r="D109" t="s">
-        <v>258</v>
-      </c>
-      <c r="E109" t="s">
-        <v>260</v>
       </c>
       <c r="F109" t="s">
         <v>6</v>
@@ -3569,19 +3569,19 @@
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
+        <v>260</v>
+      </c>
+      <c r="B110" t="s">
+        <v>125</v>
+      </c>
+      <c r="C110" t="s">
+        <v>250</v>
+      </c>
+      <c r="D110" t="s">
         <v>261</v>
       </c>
-      <c r="B110" t="s">
-        <v>126</v>
-      </c>
-      <c r="C110" t="s">
-        <v>251</v>
-      </c>
-      <c r="D110" t="s">
-        <v>262</v>
-      </c>
       <c r="E110" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="F110" t="s">
         <v>6</v>
@@ -3589,19 +3589,19 @@
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
+        <v>262</v>
+      </c>
+      <c r="B111" t="s">
+        <v>125</v>
+      </c>
+      <c r="C111" t="s">
+        <v>250</v>
+      </c>
+      <c r="D111" t="s">
         <v>263</v>
       </c>
-      <c r="B111" t="s">
-        <v>126</v>
-      </c>
-      <c r="C111" t="s">
-        <v>251</v>
-      </c>
-      <c r="D111" t="s">
-        <v>264</v>
-      </c>
       <c r="E111" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="F111" t="s">
         <v>6</v>
@@ -3609,19 +3609,19 @@
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
+        <v>264</v>
+      </c>
+      <c r="B112" t="s">
+        <v>125</v>
+      </c>
+      <c r="C112" t="s">
+        <v>250</v>
+      </c>
+      <c r="D112" t="s">
         <v>265</v>
       </c>
-      <c r="B112" t="s">
-        <v>126</v>
-      </c>
-      <c r="C112" t="s">
-        <v>251</v>
-      </c>
-      <c r="D112" t="s">
-        <v>266</v>
-      </c>
       <c r="E112" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="F112" t="s">
         <v>6</v>
@@ -3629,19 +3629,19 @@
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B113" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C113" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="D113" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="E113" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="F113" t="s">
         <v>6</v>
@@ -3649,19 +3649,19 @@
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
+        <v>267</v>
+      </c>
+      <c r="B114" t="s">
+        <v>125</v>
+      </c>
+      <c r="C114" t="s">
+        <v>250</v>
+      </c>
+      <c r="D114" t="s">
         <v>268</v>
       </c>
-      <c r="B114" t="s">
-        <v>126</v>
-      </c>
-      <c r="C114" t="s">
-        <v>251</v>
-      </c>
-      <c r="D114" t="s">
-        <v>269</v>
-      </c>
       <c r="E114" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="F114" t="s">
         <v>6</v>
@@ -3669,19 +3669,19 @@
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
+        <v>274</v>
+      </c>
+      <c r="B115" t="s">
+        <v>270</v>
+      </c>
+      <c r="C115" t="s">
+        <v>26</v>
+      </c>
+      <c r="D115" t="s">
         <v>275</v>
       </c>
-      <c r="B115" t="s">
+      <c r="E115" t="s">
         <v>271</v>
-      </c>
-      <c r="C115" t="s">
-        <v>27</v>
-      </c>
-      <c r="D115" t="s">
-        <v>276</v>
-      </c>
-      <c r="E115" t="s">
-        <v>272</v>
       </c>
       <c r="F115" t="s">
         <v>6</v>
@@ -3689,19 +3689,19 @@
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B116" t="s">
+        <v>270</v>
+      </c>
+      <c r="C116" t="s">
+        <v>26</v>
+      </c>
+      <c r="D116" t="s">
+        <v>276</v>
+      </c>
+      <c r="E116" t="s">
         <v>271</v>
-      </c>
-      <c r="C116" t="s">
-        <v>27</v>
-      </c>
-      <c r="D116" t="s">
-        <v>277</v>
-      </c>
-      <c r="E116" t="s">
-        <v>272</v>
       </c>
       <c r="F116" t="s">
         <v>6</v>
@@ -3709,19 +3709,19 @@
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B117" t="s">
+        <v>270</v>
+      </c>
+      <c r="C117" t="s">
+        <v>26</v>
+      </c>
+      <c r="D117" t="s">
+        <v>277</v>
+      </c>
+      <c r="E117" t="s">
         <v>271</v>
-      </c>
-      <c r="C117" t="s">
-        <v>27</v>
-      </c>
-      <c r="D117" t="s">
-        <v>278</v>
-      </c>
-      <c r="E117" t="s">
-        <v>272</v>
       </c>
       <c r="F117" t="s">
         <v>6</v>
@@ -3729,19 +3729,19 @@
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B118" t="s">
+        <v>279</v>
+      </c>
+      <c r="C118" t="s">
+        <v>295</v>
+      </c>
+      <c r="D118" t="s">
         <v>280</v>
       </c>
-      <c r="C118" t="s">
-        <v>296</v>
-      </c>
-      <c r="D118" t="s">
-        <v>281</v>
-      </c>
       <c r="E118" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F118" t="s">
         <v>6</v>
@@ -3749,19 +3749,19 @@
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B119" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C119" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="D119" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="E119" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F119" t="s">
         <v>6</v>
@@ -3769,19 +3769,19 @@
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
+        <v>283</v>
+      </c>
+      <c r="B120" t="s">
+        <v>279</v>
+      </c>
+      <c r="C120" t="s">
+        <v>295</v>
+      </c>
+      <c r="D120" t="s">
         <v>284</v>
       </c>
-      <c r="B120" t="s">
-        <v>280</v>
-      </c>
-      <c r="C120" t="s">
-        <v>296</v>
-      </c>
-      <c r="D120" t="s">
-        <v>285</v>
-      </c>
       <c r="E120" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F120" t="s">
         <v>6</v>
@@ -3789,19 +3789,19 @@
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B121" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C121" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="D121" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="E121" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F121" t="s">
         <v>6</v>
@@ -3809,19 +3809,19 @@
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B122" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C122" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="D122" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="E122" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F122" t="s">
         <v>6</v>
@@ -3829,19 +3829,19 @@
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
+        <v>289</v>
+      </c>
+      <c r="B123" t="s">
+        <v>279</v>
+      </c>
+      <c r="C123" t="s">
+        <v>295</v>
+      </c>
+      <c r="D123" t="s">
         <v>290</v>
       </c>
-      <c r="B123" t="s">
-        <v>280</v>
-      </c>
-      <c r="C123" t="s">
-        <v>296</v>
-      </c>
-      <c r="D123" t="s">
-        <v>291</v>
-      </c>
       <c r="E123" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F123" t="s">
         <v>6</v>
@@ -3849,19 +3849,19 @@
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
+        <v>291</v>
+      </c>
+      <c r="B124" t="s">
+        <v>279</v>
+      </c>
+      <c r="C124" t="s">
+        <v>295</v>
+      </c>
+      <c r="D124" t="s">
         <v>292</v>
       </c>
-      <c r="B124" t="s">
-        <v>280</v>
-      </c>
-      <c r="C124" t="s">
-        <v>296</v>
-      </c>
-      <c r="D124" t="s">
+      <c r="E124" t="s">
         <v>293</v>
-      </c>
-      <c r="E124" t="s">
-        <v>294</v>
       </c>
       <c r="F124" t="s">
         <v>6</v>
@@ -3869,162 +3869,162 @@
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
+        <v>301</v>
+      </c>
+      <c r="B125" t="s">
         <v>302</v>
-      </c>
-      <c r="B125" t="s">
-        <v>303</v>
       </c>
       <c r="C125" t="s">
         <v>7</v>
       </c>
       <c r="D125" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="E125" t="s">
+        <v>303</v>
+      </c>
+      <c r="F125" t="s">
         <v>304</v>
-      </c>
-      <c r="F125" t="s">
-        <v>305</v>
       </c>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B126" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C126" t="s">
         <v>7</v>
       </c>
       <c r="D126" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="E126" t="s">
+        <v>303</v>
+      </c>
+      <c r="F126" t="s">
         <v>304</v>
-      </c>
-      <c r="F126" t="s">
-        <v>305</v>
       </c>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B127" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C127" t="s">
         <v>7</v>
       </c>
       <c r="D127" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="E127" t="s">
+        <v>303</v>
+      </c>
+      <c r="F127" t="s">
         <v>304</v>
-      </c>
-      <c r="F127" t="s">
-        <v>305</v>
       </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="B128" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C128" t="s">
         <v>7</v>
       </c>
       <c r="D128" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="E128" t="s">
+        <v>303</v>
+      </c>
+      <c r="F128" t="s">
         <v>304</v>
-      </c>
-      <c r="F128" t="s">
-        <v>305</v>
       </c>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="B129" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C129" t="s">
         <v>7</v>
       </c>
       <c r="D129" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="E129" t="s">
+        <v>303</v>
+      </c>
+      <c r="F129" t="s">
         <v>304</v>
-      </c>
-      <c r="F129" t="s">
-        <v>305</v>
       </c>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="B130" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C130" t="s">
         <v>7</v>
       </c>
       <c r="D130" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="E130" t="s">
+        <v>303</v>
+      </c>
+      <c r="F130" t="s">
         <v>304</v>
-      </c>
-      <c r="F130" t="s">
-        <v>305</v>
       </c>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="B131" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C131" t="s">
         <v>7</v>
       </c>
       <c r="D131" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="E131" t="s">
+        <v>303</v>
+      </c>
+      <c r="F131" t="s">
         <v>304</v>
-      </c>
-      <c r="F131" t="s">
-        <v>305</v>
       </c>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B132" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C132" t="s">
         <v>7</v>
       </c>
       <c r="D132" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="E132" t="s">
+        <v>303</v>
+      </c>
+      <c r="F132" t="s">
         <v>304</v>
-      </c>
-      <c r="F132" t="s">
-        <v>305</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Katalog guncellendi - 15.07.2026 17:17:03,71
</commit_message>
<xml_diff>
--- a/urunler.xlsx
+++ b/urunler.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/49dd5535ee0ab452/Desktop/YEMEK LİSTELERİ/yemek/CEREN-PC/SIVAL_GIYIM_KATALOG/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="214" documentId="13_ncr:1_{CCE8B614-DB69-4334-AC06-D714AC841E42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{50ABA224-DFB3-445E-B080-66A8B0F3AEEA}"/>
+  <xr:revisionPtr revIDLastSave="220" documentId="13_ncr:1_{CCE8B614-DB69-4334-AC06-D714AC841E42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{57E72589-8F78-4432-B708-12E9263E1BD1}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="792" uniqueCount="321">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="797" uniqueCount="325">
   <si>
     <t>urun_adi</t>
   </si>
@@ -983,6 +983,18 @@
   </si>
   <si>
     <t>350 Tl</t>
+  </si>
+  <si>
+    <t>MASTİF 824 TŞÖRT</t>
+  </si>
+  <si>
+    <t>300 TL</t>
+  </si>
+  <si>
+    <t>Tşört</t>
+  </si>
+  <si>
+    <t>WhatsApp Image 2026-07-15 at 17.11.36.jpg</t>
   </si>
 </sst>
 </file>
@@ -1379,7 +1391,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F132"/>
+  <dimension ref="A1:F133"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="52.28515625" customWidth="1"/>
@@ -4027,6 +4039,23 @@
         <v>304</v>
       </c>
     </row>
+    <row r="133" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A133" t="s">
+        <v>321</v>
+      </c>
+      <c r="B133" t="s">
+        <v>322</v>
+      </c>
+      <c r="C133" t="s">
+        <v>323</v>
+      </c>
+      <c r="D133" t="s">
+        <v>324</v>
+      </c>
+      <c r="E133" t="s">
+        <v>271</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Katalog guncellendi - 15.07.2026 17:19:07,38
</commit_message>
<xml_diff>
--- a/urunler.xlsx
+++ b/urunler.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/49dd5535ee0ab452/Desktop/YEMEK LİSTELERİ/yemek/CEREN-PC/SIVAL_GIYIM_KATALOG/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="220" documentId="13_ncr:1_{CCE8B614-DB69-4334-AC06-D714AC841E42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{57E72589-8F78-4432-B708-12E9263E1BD1}"/>
+  <xr:revisionPtr revIDLastSave="223" documentId="13_ncr:1_{CCE8B614-DB69-4334-AC06-D714AC841E42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E9FCB3CD-808B-4B04-A28A-8B7F9A1942DD}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -994,7 +994,7 @@
     <t>Tşört</t>
   </si>
   <si>
-    <t>WhatsApp Image 2026-07-15 at 17.11.36.jpg</t>
+    <t>kahvetşörtt.jpg</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Katalog guncellendi - 15.07.2026 17:23:37,88
</commit_message>
<xml_diff>
--- a/urunler.xlsx
+++ b/urunler.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/49dd5535ee0ab452/Desktop/YEMEK LİSTELERİ/yemek/CEREN-PC/SIVAL_GIYIM_KATALOG/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="224" documentId="13_ncr:1_{CCE8B614-DB69-4334-AC06-D714AC841E42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5F808405-5B0C-4ABC-B225-E9BB5AF68A5F}"/>
+  <xr:revisionPtr revIDLastSave="226" documentId="13_ncr:1_{CCE8B614-DB69-4334-AC06-D714AC841E42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AE2E44ED-BE0D-40C7-8A01-EE9C1134E0BB}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -994,7 +994,7 @@
     <t>Tşört</t>
   </si>
   <si>
-    <t>kahvetşörtt.jpg</t>
+    <t>KAHVET.jpg</t>
   </si>
 </sst>
 </file>
@@ -4053,7 +4053,7 @@
         <v>324</v>
       </c>
       <c r="E133" t="s">
-        <v>271</v>
+        <v>259</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Katalog guncellendi - 15.07.2026 17:32:19,77
</commit_message>
<xml_diff>
--- a/urunler.xlsx
+++ b/urunler.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/49dd5535ee0ab452/Desktop/YEMEK LİSTELERİ/yemek/CEREN-PC/SIVAL_GIYIM_KATALOG/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="226" documentId="13_ncr:1_{CCE8B614-DB69-4334-AC06-D714AC841E42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AE2E44ED-BE0D-40C7-8A01-EE9C1134E0BB}"/>
+  <xr:revisionPtr revIDLastSave="227" documentId="13_ncr:1_{CCE8B614-DB69-4334-AC06-D714AC841E42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{32542729-8EAA-4D92-B725-8B4C153D7932}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="797" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="828" uniqueCount="335">
   <si>
     <t>urun_adi</t>
   </si>
@@ -985,9 +985,6 @@
     <t>350 Tl</t>
   </si>
   <si>
-    <t>MASTİF 824 TŞÖRT</t>
-  </si>
-  <si>
     <t>300 TL</t>
   </si>
   <si>
@@ -995,6 +992,39 @@
   </si>
   <si>
     <t>KAHVET.jpg</t>
+  </si>
+  <si>
+    <t>MASTİF 824 TŞÖRT KAHVERENGİ</t>
+  </si>
+  <si>
+    <t>MASTİF 824 TŞÖRT SİYAH</t>
+  </si>
+  <si>
+    <t>SİYAHT.jpg</t>
+  </si>
+  <si>
+    <t>MASTİF 824 TŞÖRT GRİ</t>
+  </si>
+  <si>
+    <t>GRİT.jpg</t>
+  </si>
+  <si>
+    <t>MASTİF 824 TŞÖRT KREM</t>
+  </si>
+  <si>
+    <t>KREMT.jpg</t>
+  </si>
+  <si>
+    <t>MASTİF 824 TŞÖRT LACİVERT</t>
+  </si>
+  <si>
+    <t>LACİT.jpg</t>
+  </si>
+  <si>
+    <t>MASTİF 824 TŞÖRT BEYAZ</t>
+  </si>
+  <si>
+    <t>BEYAZT.jpg</t>
   </si>
 </sst>
 </file>
@@ -1391,7 +1421,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F133"/>
+  <dimension ref="A1:F138"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="52.28515625" customWidth="1"/>
@@ -4041,19 +4071,122 @@
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
+        <v>324</v>
+      </c>
+      <c r="B133" t="s">
         <v>321</v>
       </c>
-      <c r="B133" t="s">
+      <c r="C133" t="s">
         <v>322</v>
       </c>
-      <c r="C133" t="s">
+      <c r="D133" t="s">
         <v>323</v>
-      </c>
-      <c r="D133" t="s">
-        <v>324</v>
       </c>
       <c r="E133" t="s">
         <v>259</v>
+      </c>
+      <c r="F133" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="134" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A134" t="s">
+        <v>325</v>
+      </c>
+      <c r="B134" t="s">
+        <v>321</v>
+      </c>
+      <c r="C134" t="s">
+        <v>322</v>
+      </c>
+      <c r="D134" t="s">
+        <v>326</v>
+      </c>
+      <c r="E134" t="s">
+        <v>259</v>
+      </c>
+      <c r="F134" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="135" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A135" t="s">
+        <v>327</v>
+      </c>
+      <c r="B135" t="s">
+        <v>321</v>
+      </c>
+      <c r="C135" t="s">
+        <v>322</v>
+      </c>
+      <c r="D135" t="s">
+        <v>328</v>
+      </c>
+      <c r="E135" t="s">
+        <v>259</v>
+      </c>
+      <c r="F135" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="136" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A136" t="s">
+        <v>329</v>
+      </c>
+      <c r="B136" t="s">
+        <v>321</v>
+      </c>
+      <c r="C136" t="s">
+        <v>322</v>
+      </c>
+      <c r="D136" t="s">
+        <v>330</v>
+      </c>
+      <c r="E136" t="s">
+        <v>259</v>
+      </c>
+      <c r="F136" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="137" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A137" t="s">
+        <v>331</v>
+      </c>
+      <c r="B137" t="s">
+        <v>321</v>
+      </c>
+      <c r="C137" t="s">
+        <v>322</v>
+      </c>
+      <c r="D137" t="s">
+        <v>332</v>
+      </c>
+      <c r="E137" t="s">
+        <v>259</v>
+      </c>
+      <c r="F137" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="138" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A138" t="s">
+        <v>333</v>
+      </c>
+      <c r="B138" t="s">
+        <v>321</v>
+      </c>
+      <c r="C138" t="s">
+        <v>322</v>
+      </c>
+      <c r="D138" t="s">
+        <v>334</v>
+      </c>
+      <c r="E138" t="s">
+        <v>259</v>
+      </c>
+      <c r="F138" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Katalog guncellendi - 16.07.2026  9:27:21,18
</commit_message>
<xml_diff>
--- a/urunler.xlsx
+++ b/urunler.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/49dd5535ee0ab452/Desktop/YEMEK LİSTELERİ/yemek/CEREN-PC/SIVAL_GIYIM_KATALOG/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="227" documentId="13_ncr:1_{CCE8B614-DB69-4334-AC06-D714AC841E42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{32542729-8EAA-4D92-B725-8B4C153D7932}"/>
+  <xr:revisionPtr revIDLastSave="236" documentId="13_ncr:1_{CCE8B614-DB69-4334-AC06-D714AC841E42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4ACAC5F1-66BB-459A-A1A1-214E3B590D1B}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="828" uniqueCount="335">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="833" uniqueCount="339">
   <si>
     <t>urun_adi</t>
   </si>
@@ -1025,6 +1025,18 @@
   </si>
   <si>
     <t>BEYAZT.jpg</t>
+  </si>
+  <si>
+    <t>MASTİFF 4522 BATTAL TŞÖRT</t>
+  </si>
+  <si>
+    <t>265TL</t>
+  </si>
+  <si>
+    <t>battal.jpg</t>
+  </si>
+  <si>
+    <t>2XL-3XL-4XL-5XL-6XL Beden seçeneği mevcuttur.Ürünümüz serili olarak satılmaktadır.Belirtilen fiyatlar adet fiyatıdır.</t>
   </si>
 </sst>
 </file>
@@ -1421,7 +1433,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F138"/>
+  <dimension ref="A1:F139"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="52.28515625" customWidth="1"/>
@@ -4189,6 +4201,23 @@
         <v>6</v>
       </c>
     </row>
+    <row r="139" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A139" t="s">
+        <v>335</v>
+      </c>
+      <c r="B139" t="s">
+        <v>336</v>
+      </c>
+      <c r="C139" t="s">
+        <v>322</v>
+      </c>
+      <c r="D139" t="s">
+        <v>337</v>
+      </c>
+      <c r="E139" t="s">
+        <v>338</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Katalog guncellendi - 16.07.2026  9:34:10,26
</commit_message>
<xml_diff>
--- a/urunler.xlsx
+++ b/urunler.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/49dd5535ee0ab452/Desktop/YEMEK LİSTELERİ/yemek/CEREN-PC/SIVAL_GIYIM_KATALOG/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="236" documentId="13_ncr:1_{CCE8B614-DB69-4334-AC06-D714AC841E42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4ACAC5F1-66BB-459A-A1A1-214E3B590D1B}"/>
+  <xr:revisionPtr revIDLastSave="241" documentId="13_ncr:1_{CCE8B614-DB69-4334-AC06-D714AC841E42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1DFAF219-C068-4AC0-864D-7361BE7CBE0E}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="833" uniqueCount="339">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="838" uniqueCount="342">
   <si>
     <t>urun_adi</t>
   </si>
@@ -1037,6 +1037,15 @@
   </si>
   <si>
     <t>2XL-3XL-4XL-5XL-6XL Beden seçeneği mevcuttur.Ürünümüz serili olarak satılmaktadır.Belirtilen fiyatlar adet fiyatıdır.</t>
+  </si>
+  <si>
+    <t>SIFIRKOL.jpg</t>
+  </si>
+  <si>
+    <t>MUSİC SIFIR KOL TŞÖRT</t>
+  </si>
+  <si>
+    <t>140 TL</t>
   </si>
 </sst>
 </file>
@@ -1433,7 +1442,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F139"/>
+  <dimension ref="A1:F140"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="52.28515625" customWidth="1"/>
@@ -4218,6 +4227,23 @@
         <v>338</v>
       </c>
     </row>
+    <row r="140" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A140" t="s">
+        <v>340</v>
+      </c>
+      <c r="B140" t="s">
+        <v>341</v>
+      </c>
+      <c r="C140" t="s">
+        <v>322</v>
+      </c>
+      <c r="D140" t="s">
+        <v>339</v>
+      </c>
+      <c r="E140" t="s">
+        <v>259</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Katalog guncellendi - 16.07.2026  9:38:13,89
</commit_message>
<xml_diff>
--- a/urunler.xlsx
+++ b/urunler.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/49dd5535ee0ab452/Desktop/YEMEK LİSTELERİ/yemek/CEREN-PC/SIVAL_GIYIM_KATALOG/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="241" documentId="13_ncr:1_{CCE8B614-DB69-4334-AC06-D714AC841E42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1DFAF219-C068-4AC0-864D-7361BE7CBE0E}"/>
+  <xr:revisionPtr revIDLastSave="242" documentId="13_ncr:1_{CCE8B614-DB69-4334-AC06-D714AC841E42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6CF9DD76-3C18-4C1A-AE09-9EDEC50570C3}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1039,13 +1039,13 @@
     <t>2XL-3XL-4XL-5XL-6XL Beden seçeneği mevcuttur.Ürünümüz serili olarak satılmaktadır.Belirtilen fiyatlar adet fiyatıdır.</t>
   </si>
   <si>
-    <t>SIFIRKOL.jpg</t>
-  </si>
-  <si>
     <t>MUSİC SIFIR KOL TŞÖRT</t>
   </si>
   <si>
     <t>140 TL</t>
+  </si>
+  <si>
+    <t>sıfırkol.jpg</t>
   </si>
 </sst>
 </file>
@@ -4229,16 +4229,16 @@
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
+        <v>339</v>
+      </c>
+      <c r="B140" t="s">
         <v>340</v>
-      </c>
-      <c r="B140" t="s">
-        <v>341</v>
       </c>
       <c r="C140" t="s">
         <v>322</v>
       </c>
       <c r="D140" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="E140" t="s">
         <v>259</v>

</xml_diff>

<commit_message>
Katalog guncellendi - 16.07.2026  9:40:06,08
</commit_message>
<xml_diff>
--- a/urunler.xlsx
+++ b/urunler.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/49dd5535ee0ab452/Desktop/YEMEK LİSTELERİ/yemek/CEREN-PC/SIVAL_GIYIM_KATALOG/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="242" documentId="13_ncr:1_{CCE8B614-DB69-4334-AC06-D714AC841E42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6CF9DD76-3C18-4C1A-AE09-9EDEC50570C3}"/>
+  <xr:revisionPtr revIDLastSave="249" documentId="13_ncr:1_{CCE8B614-DB69-4334-AC06-D714AC841E42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3966369C-27F2-48D3-A59A-064C36BC7489}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="838" uniqueCount="342">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="844" uniqueCount="345">
   <si>
     <t>urun_adi</t>
   </si>
@@ -1046,6 +1046,15 @@
   </si>
   <si>
     <t>sıfırkol.jpg</t>
+  </si>
+  <si>
+    <t>MUSİC POLYESTER TŞÖRT</t>
+  </si>
+  <si>
+    <t>155 TL</t>
+  </si>
+  <si>
+    <t>ÇİZGİLİ.JPG</t>
   </si>
 </sst>
 </file>
@@ -1442,7 +1451,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F140"/>
+  <dimension ref="A1:F141"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="52.28515625" customWidth="1"/>
@@ -4226,6 +4235,9 @@
       <c r="E139" t="s">
         <v>338</v>
       </c>
+      <c r="F139" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
@@ -4242,6 +4254,23 @@
       </c>
       <c r="E140" t="s">
         <v>259</v>
+      </c>
+      <c r="F140" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="141" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A141" t="s">
+        <v>342</v>
+      </c>
+      <c r="B141" t="s">
+        <v>343</v>
+      </c>
+      <c r="C141" t="s">
+        <v>322</v>
+      </c>
+      <c r="D141" t="s">
+        <v>344</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Katalog guncellendi - 16.07.2026  9:42:01,14
</commit_message>
<xml_diff>
--- a/urunler.xlsx
+++ b/urunler.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/49dd5535ee0ab452/Desktop/YEMEK LİSTELERİ/yemek/CEREN-PC/SIVAL_GIYIM_KATALOG/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="249" documentId="13_ncr:1_{CCE8B614-DB69-4334-AC06-D714AC841E42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3966369C-27F2-48D3-A59A-064C36BC7489}"/>
+  <xr:revisionPtr revIDLastSave="260" documentId="13_ncr:1_{CCE8B614-DB69-4334-AC06-D714AC841E42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2690A2FC-DBF6-490D-9615-55D58AD8AB3D}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="844" uniqueCount="345">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="852" uniqueCount="347">
   <si>
     <t>urun_adi</t>
   </si>
@@ -1054,7 +1054,13 @@
     <t>155 TL</t>
   </si>
   <si>
-    <t>ÇİZGİLİ.JPG</t>
+    <t>MASTİF 841 TŞÖRT</t>
+  </si>
+  <si>
+    <t>ÇİZGİLİ.jpg</t>
+  </si>
+  <si>
+    <t>841.jpg</t>
   </si>
 </sst>
 </file>
@@ -1451,7 +1457,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F141"/>
+  <dimension ref="A1:F142"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="52.28515625" customWidth="1"/>
@@ -4270,7 +4276,33 @@
         <v>322</v>
       </c>
       <c r="D141" t="s">
+        <v>345</v>
+      </c>
+      <c r="E141" t="s">
+        <v>259</v>
+      </c>
+      <c r="F141" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="142" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A142" t="s">
         <v>344</v>
+      </c>
+      <c r="B142" t="s">
+        <v>321</v>
+      </c>
+      <c r="C142" t="s">
+        <v>322</v>
+      </c>
+      <c r="D142" t="s">
+        <v>346</v>
+      </c>
+      <c r="E142" t="s">
+        <v>259</v>
+      </c>
+      <c r="F142" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Katalog guncellendi - 16.07.2026  9:44:01,00
</commit_message>
<xml_diff>
--- a/urunler.xlsx
+++ b/urunler.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/49dd5535ee0ab452/Desktop/YEMEK LİSTELERİ/yemek/CEREN-PC/SIVAL_GIYIM_KATALOG/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="260" documentId="13_ncr:1_{CCE8B614-DB69-4334-AC06-D714AC841E42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2690A2FC-DBF6-490D-9615-55D58AD8AB3D}"/>
+  <xr:revisionPtr revIDLastSave="261" documentId="13_ncr:1_{CCE8B614-DB69-4334-AC06-D714AC841E42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B27F7406-51B3-45C1-BFA2-E306624287D4}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1060,7 +1060,7 @@
     <t>ÇİZGİLİ.jpg</t>
   </si>
   <si>
-    <t>841.jpg</t>
+    <t>MASTİF841.jpg</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Katalog guncellendi - 16.07.2026  9:48:14,59
</commit_message>
<xml_diff>
--- a/urunler.xlsx
+++ b/urunler.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/49dd5535ee0ab452/Desktop/YEMEK LİSTELERİ/yemek/CEREN-PC/SIVAL_GIYIM_KATALOG/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="261" documentId="13_ncr:1_{CCE8B614-DB69-4334-AC06-D714AC841E42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B27F7406-51B3-45C1-BFA2-E306624287D4}"/>
+  <xr:revisionPtr revIDLastSave="263" documentId="13_ncr:1_{CCE8B614-DB69-4334-AC06-D714AC841E42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0418AB1C-B777-4FD3-A8D4-C207CB7EBE3B}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1060,7 +1060,7 @@
     <t>ÇİZGİLİ.jpg</t>
   </si>
   <si>
-    <t>MASTİF841.jpg</t>
+    <t>MASTİFF.jpg</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Katalog guncellendi - 16.07.2026 10:04:49,34
</commit_message>
<xml_diff>
--- a/urunler.xlsx
+++ b/urunler.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/49dd5535ee0ab452/Desktop/YEMEK LİSTELERİ/yemek/CEREN-PC/SIVAL_GIYIM_KATALOG/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="263" documentId="13_ncr:1_{CCE8B614-DB69-4334-AC06-D714AC841E42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0418AB1C-B777-4FD3-A8D4-C207CB7EBE3B}"/>
+  <xr:revisionPtr revIDLastSave="283" documentId="13_ncr:1_{CCE8B614-DB69-4334-AC06-D714AC841E42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ED5F4FA8-0CD4-4F1D-BF88-706846A9ACC5}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="852" uniqueCount="347">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="876" uniqueCount="353">
   <si>
     <t>urun_adi</t>
   </si>
@@ -1061,6 +1061,24 @@
   </si>
   <si>
     <t>MASTİFF.jpg</t>
+  </si>
+  <si>
+    <t>KISA KIL ÇITÇITLI GÖMLEK</t>
+  </si>
+  <si>
+    <t>245 TL</t>
+  </si>
+  <si>
+    <t>kısakolgg.jpg</t>
+  </si>
+  <si>
+    <t>kısakolg.jpg</t>
+  </si>
+  <si>
+    <t>kısakolgk.jpg</t>
+  </si>
+  <si>
+    <t>kısakolgb.jpg</t>
   </si>
 </sst>
 </file>
@@ -1457,7 +1475,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F142"/>
+  <dimension ref="A1:F146"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="52.28515625" customWidth="1"/>
@@ -4305,6 +4323,86 @@
         <v>6</v>
       </c>
     </row>
+    <row r="143" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A143" t="s">
+        <v>347</v>
+      </c>
+      <c r="B143" t="s">
+        <v>348</v>
+      </c>
+      <c r="C143" t="s">
+        <v>26</v>
+      </c>
+      <c r="D143" t="s">
+        <v>350</v>
+      </c>
+      <c r="E143" t="s">
+        <v>259</v>
+      </c>
+      <c r="F143" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="144" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A144" t="s">
+        <v>347</v>
+      </c>
+      <c r="B144" t="s">
+        <v>348</v>
+      </c>
+      <c r="C144" t="s">
+        <v>26</v>
+      </c>
+      <c r="D144" t="s">
+        <v>349</v>
+      </c>
+      <c r="E144" t="s">
+        <v>259</v>
+      </c>
+      <c r="F144" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="145" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A145" t="s">
+        <v>347</v>
+      </c>
+      <c r="B145" t="s">
+        <v>348</v>
+      </c>
+      <c r="C145" t="s">
+        <v>26</v>
+      </c>
+      <c r="D145" t="s">
+        <v>351</v>
+      </c>
+      <c r="E145" t="s">
+        <v>259</v>
+      </c>
+      <c r="F145" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="146" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A146" t="s">
+        <v>347</v>
+      </c>
+      <c r="B146" t="s">
+        <v>348</v>
+      </c>
+      <c r="C146" t="s">
+        <v>26</v>
+      </c>
+      <c r="D146" t="s">
+        <v>352</v>
+      </c>
+      <c r="E146" t="s">
+        <v>259</v>
+      </c>
+      <c r="F146" t="s">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Katalog guncellendi - 16.07.2026 10:23:36,99
</commit_message>
<xml_diff>
--- a/urunler.xlsx
+++ b/urunler.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/49dd5535ee0ab452/Desktop/YEMEK LİSTELERİ/yemek/CEREN-PC/SIVAL_GIYIM_KATALOG/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="283" documentId="13_ncr:1_{CCE8B614-DB69-4334-AC06-D714AC841E42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ED5F4FA8-0CD4-4F1D-BF88-706846A9ACC5}"/>
+  <xr:revisionPtr revIDLastSave="288" documentId="13_ncr:1_{CCE8B614-DB69-4334-AC06-D714AC841E42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A9BCE2C2-BB09-46E5-A987-42F30348410E}"/>
   <bookViews>
     <workbookView xWindow="7200" yWindow="4185" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1063,9 +1063,6 @@
     <t>MASTİFF.jpg</t>
   </si>
   <si>
-    <t>KISA KIL ÇITÇITLI GÖMLEK</t>
-  </si>
-  <si>
     <t>245 TL</t>
   </si>
   <si>
@@ -1078,7 +1075,10 @@
     <t>kısakolgk.jpg</t>
   </si>
   <si>
-    <t>kısakolgb.jpg</t>
+    <t>KISA KOL ÇITÇITLI GÖMLEK</t>
+  </si>
+  <si>
+    <t>KISAKOLGB.jpg</t>
   </si>
 </sst>
 </file>
@@ -4325,16 +4325,16 @@
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
+        <v>351</v>
+      </c>
+      <c r="B143" t="s">
         <v>347</v>
-      </c>
-      <c r="B143" t="s">
-        <v>348</v>
       </c>
       <c r="C143" t="s">
         <v>26</v>
       </c>
       <c r="D143" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="E143" t="s">
         <v>259</v>
@@ -4345,16 +4345,16 @@
     </row>
     <row r="144" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
+        <v>351</v>
+      </c>
+      <c r="B144" t="s">
         <v>347</v>
-      </c>
-      <c r="B144" t="s">
-        <v>348</v>
       </c>
       <c r="C144" t="s">
         <v>26</v>
       </c>
       <c r="D144" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="E144" t="s">
         <v>259</v>
@@ -4365,16 +4365,16 @@
     </row>
     <row r="145" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
+        <v>351</v>
+      </c>
+      <c r="B145" t="s">
         <v>347</v>
-      </c>
-      <c r="B145" t="s">
-        <v>348</v>
       </c>
       <c r="C145" t="s">
         <v>26</v>
       </c>
       <c r="D145" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="E145" t="s">
         <v>259</v>
@@ -4385,10 +4385,10 @@
     </row>
     <row r="146" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
+        <v>351</v>
+      </c>
+      <c r="B146" t="s">
         <v>347</v>
-      </c>
-      <c r="B146" t="s">
-        <v>348</v>
       </c>
       <c r="C146" t="s">
         <v>26</v>

</xml_diff>

<commit_message>
Katalog guncellendi - 16.07.2026 10:25:07,01
</commit_message>
<xml_diff>
--- a/urunler.xlsx
+++ b/urunler.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/49dd5535ee0ab452/Desktop/YEMEK LİSTELERİ/yemek/CEREN-PC/SIVAL_GIYIM_KATALOG/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="288" documentId="13_ncr:1_{CCE8B614-DB69-4334-AC06-D714AC841E42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A9BCE2C2-BB09-46E5-A987-42F30348410E}"/>
+  <xr:revisionPtr revIDLastSave="289" documentId="13_ncr:1_{CCE8B614-DB69-4334-AC06-D714AC841E42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CD1C3B3A-C408-41AE-944D-34992CDA07ED}"/>
   <bookViews>
     <workbookView xWindow="7200" yWindow="4185" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="876" uniqueCount="353">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="876" uniqueCount="354">
   <si>
     <t>urun_adi</t>
   </si>
@@ -1079,6 +1079,9 @@
   </si>
   <si>
     <t>KISAKOLGB.jpg</t>
+  </si>
+  <si>
+    <t>gömlek</t>
   </si>
 </sst>
 </file>
@@ -4391,7 +4394,7 @@
         <v>347</v>
       </c>
       <c r="C146" t="s">
-        <v>26</v>
+        <v>353</v>
       </c>
       <c r="D146" t="s">
         <v>352</v>

</xml_diff>